<commit_message>
feat(planas): update Excel template 1-INF.-N-000-26-AG34-PLANAS-ASTM-D4791-V02-1-M.xlsx
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/Planas/1-INF.-N-000-26-AG34-PLANAS-ASTM-D4791-V02-1-M.xlsx
+++ b/app/templates/informes/Informes agregado/Planas/1-INF.-N-000-26-AG34-PLANAS-ASTM-D4791-V02-1-M.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.2 Informe agregados\INFORME ACREDITADO-E ISO\1.1 JUNIO 15-06-26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\Planas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5472F1E0-A0BB-4F86-9ADF-15FCFDE1C648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125C8B28-FA09-4392-8F62-37E4897C61DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="641" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="641" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="97" r:id="rId1"/>
@@ -3279,6 +3279,9 @@
     <xf numFmtId="174" fontId="28" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3352,12 +3355,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="8" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="54" fillId="0" borderId="9" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="54" fillId="0" borderId="8" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3920,13 +3917,16 @@
     <xf numFmtId="0" fontId="28" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="182" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="183" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="9" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="8" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4179,7 +4179,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145561856"/>
@@ -4215,7 +4215,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145560320"/>
@@ -4253,7 +4253,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4411,7 +4411,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145561856"/>
@@ -4447,7 +4447,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145560320"/>
@@ -4485,7 +4485,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4643,7 +4643,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145561856"/>
@@ -4679,7 +4679,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145560320"/>
@@ -4717,7 +4717,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4875,7 +4875,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145561856"/>
@@ -4911,7 +4911,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145560320"/>
@@ -4949,7 +4949,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -6831,7 +6831,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6890,7 +6890,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6967,7 +6967,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BGA"/>
@@ -8629,91 +8629,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="381"/>
-      <c r="B1" s="382"/>
-      <c r="C1" s="382"/>
-      <c r="D1" s="382"/>
-      <c r="E1" s="382"/>
-      <c r="F1" s="382"/>
-      <c r="G1" s="382"/>
-      <c r="H1" s="382"/>
-      <c r="I1" s="382"/>
-      <c r="J1" s="382"/>
-      <c r="K1" s="382"/>
-      <c r="L1" s="382"/>
-      <c r="M1" s="382"/>
-      <c r="N1" s="382"/>
-      <c r="O1" s="382"/>
-      <c r="P1" s="382"/>
-      <c r="Q1" s="382"/>
-      <c r="R1" s="382"/>
-      <c r="S1" s="383"/>
+      <c r="A1" s="380"/>
+      <c r="B1" s="381"/>
+      <c r="C1" s="381"/>
+      <c r="D1" s="381"/>
+      <c r="E1" s="381"/>
+      <c r="F1" s="381"/>
+      <c r="G1" s="381"/>
+      <c r="H1" s="381"/>
+      <c r="I1" s="381"/>
+      <c r="J1" s="381"/>
+      <c r="K1" s="381"/>
+      <c r="L1" s="381"/>
+      <c r="M1" s="381"/>
+      <c r="N1" s="381"/>
+      <c r="O1" s="381"/>
+      <c r="P1" s="381"/>
+      <c r="Q1" s="381"/>
+      <c r="R1" s="381"/>
+      <c r="S1" s="382"/>
       <c r="X1" s="256"/>
     </row>
     <row r="2" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="384"/>
-      <c r="B2" s="385"/>
-      <c r="C2" s="385"/>
-      <c r="D2" s="385"/>
-      <c r="E2" s="385"/>
-      <c r="F2" s="385"/>
-      <c r="G2" s="385"/>
-      <c r="H2" s="385"/>
-      <c r="I2" s="385"/>
-      <c r="J2" s="385"/>
-      <c r="K2" s="385"/>
-      <c r="L2" s="385"/>
-      <c r="M2" s="385"/>
-      <c r="N2" s="385"/>
-      <c r="O2" s="385"/>
-      <c r="P2" s="385"/>
-      <c r="Q2" s="385"/>
-      <c r="R2" s="385"/>
-      <c r="S2" s="386"/>
+      <c r="A2" s="383"/>
+      <c r="B2" s="384"/>
+      <c r="C2" s="384"/>
+      <c r="D2" s="384"/>
+      <c r="E2" s="384"/>
+      <c r="F2" s="384"/>
+      <c r="G2" s="384"/>
+      <c r="H2" s="384"/>
+      <c r="I2" s="384"/>
+      <c r="J2" s="384"/>
+      <c r="K2" s="384"/>
+      <c r="L2" s="384"/>
+      <c r="M2" s="384"/>
+      <c r="N2" s="384"/>
+      <c r="O2" s="384"/>
+      <c r="P2" s="384"/>
+      <c r="Q2" s="384"/>
+      <c r="R2" s="384"/>
+      <c r="S2" s="385"/>
       <c r="X2" s="256"/>
     </row>
     <row r="3" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="384"/>
-      <c r="B3" s="385"/>
-      <c r="C3" s="385"/>
-      <c r="D3" s="385"/>
-      <c r="E3" s="385"/>
-      <c r="F3" s="385"/>
-      <c r="G3" s="385"/>
-      <c r="H3" s="385"/>
-      <c r="I3" s="385"/>
-      <c r="J3" s="385"/>
-      <c r="K3" s="385"/>
-      <c r="L3" s="385"/>
-      <c r="M3" s="385"/>
-      <c r="N3" s="385"/>
-      <c r="O3" s="385"/>
-      <c r="P3" s="385"/>
-      <c r="Q3" s="385"/>
-      <c r="R3" s="385"/>
-      <c r="S3" s="386"/>
+      <c r="A3" s="383"/>
+      <c r="B3" s="384"/>
+      <c r="C3" s="384"/>
+      <c r="D3" s="384"/>
+      <c r="E3" s="384"/>
+      <c r="F3" s="384"/>
+      <c r="G3" s="384"/>
+      <c r="H3" s="384"/>
+      <c r="I3" s="384"/>
+      <c r="J3" s="384"/>
+      <c r="K3" s="384"/>
+      <c r="L3" s="384"/>
+      <c r="M3" s="384"/>
+      <c r="N3" s="384"/>
+      <c r="O3" s="384"/>
+      <c r="P3" s="384"/>
+      <c r="Q3" s="384"/>
+      <c r="R3" s="384"/>
+      <c r="S3" s="385"/>
       <c r="X3" s="256"/>
     </row>
     <row r="4" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="384"/>
-      <c r="B4" s="385"/>
-      <c r="C4" s="385"/>
-      <c r="D4" s="385"/>
-      <c r="E4" s="385"/>
-      <c r="F4" s="385"/>
-      <c r="G4" s="385"/>
-      <c r="H4" s="385"/>
-      <c r="I4" s="385"/>
-      <c r="J4" s="385"/>
-      <c r="K4" s="385"/>
-      <c r="L4" s="385"/>
-      <c r="M4" s="385"/>
-      <c r="N4" s="385"/>
-      <c r="O4" s="385"/>
-      <c r="P4" s="385"/>
-      <c r="Q4" s="385"/>
-      <c r="R4" s="385"/>
-      <c r="S4" s="386"/>
+      <c r="A4" s="383"/>
+      <c r="B4" s="384"/>
+      <c r="C4" s="384"/>
+      <c r="D4" s="384"/>
+      <c r="E4" s="384"/>
+      <c r="F4" s="384"/>
+      <c r="G4" s="384"/>
+      <c r="H4" s="384"/>
+      <c r="I4" s="384"/>
+      <c r="J4" s="384"/>
+      <c r="K4" s="384"/>
+      <c r="L4" s="384"/>
+      <c r="M4" s="384"/>
+      <c r="N4" s="384"/>
+      <c r="O4" s="384"/>
+      <c r="P4" s="384"/>
+      <c r="Q4" s="384"/>
+      <c r="R4" s="384"/>
+      <c r="S4" s="385"/>
       <c r="U4" s="314" t="s">
         <v>224</v>
       </c>
@@ -8721,25 +8721,25 @@
       <c r="X4" s="256"/>
     </row>
     <row r="5" spans="1:24" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="387"/>
-      <c r="B5" s="388"/>
-      <c r="C5" s="388"/>
-      <c r="D5" s="388"/>
-      <c r="E5" s="388"/>
-      <c r="F5" s="388"/>
-      <c r="G5" s="388"/>
-      <c r="H5" s="388"/>
-      <c r="I5" s="388"/>
-      <c r="J5" s="388"/>
-      <c r="K5" s="388"/>
-      <c r="L5" s="388"/>
-      <c r="M5" s="388"/>
-      <c r="N5" s="388"/>
-      <c r="O5" s="388"/>
-      <c r="P5" s="388"/>
-      <c r="Q5" s="388"/>
-      <c r="R5" s="388"/>
-      <c r="S5" s="389"/>
+      <c r="A5" s="386"/>
+      <c r="B5" s="387"/>
+      <c r="C5" s="387"/>
+      <c r="D5" s="387"/>
+      <c r="E5" s="387"/>
+      <c r="F5" s="387"/>
+      <c r="G5" s="387"/>
+      <c r="H5" s="387"/>
+      <c r="I5" s="387"/>
+      <c r="J5" s="387"/>
+      <c r="K5" s="387"/>
+      <c r="L5" s="387"/>
+      <c r="M5" s="387"/>
+      <c r="N5" s="387"/>
+      <c r="O5" s="387"/>
+      <c r="P5" s="387"/>
+      <c r="Q5" s="387"/>
+      <c r="R5" s="387"/>
+      <c r="S5" s="388"/>
       <c r="U5" s="314" t="s">
         <v>225</v>
       </c>
@@ -8753,54 +8753,54 @@
       <c r="V6" s="316"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="390" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="390"/>
-      <c r="C7" s="390"/>
-      <c r="D7" s="390"/>
-      <c r="E7" s="390"/>
-      <c r="F7" s="390"/>
-      <c r="G7" s="390"/>
-      <c r="H7" s="390"/>
-      <c r="I7" s="390"/>
-      <c r="J7" s="390"/>
-      <c r="K7" s="390"/>
-      <c r="L7" s="390"/>
-      <c r="M7" s="390"/>
-      <c r="N7" s="390"/>
-      <c r="O7" s="390"/>
-      <c r="P7" s="390"/>
-      <c r="Q7" s="390"/>
-      <c r="R7" s="390"/>
-      <c r="S7" s="390"/>
+      <c r="A7" s="389" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="389"/>
+      <c r="C7" s="389"/>
+      <c r="D7" s="389"/>
+      <c r="E7" s="389"/>
+      <c r="F7" s="389"/>
+      <c r="G7" s="389"/>
+      <c r="H7" s="389"/>
+      <c r="I7" s="389"/>
+      <c r="J7" s="389"/>
+      <c r="K7" s="389"/>
+      <c r="L7" s="389"/>
+      <c r="M7" s="389"/>
+      <c r="N7" s="389"/>
+      <c r="O7" s="389"/>
+      <c r="P7" s="389"/>
+      <c r="Q7" s="389"/>
+      <c r="R7" s="389"/>
+      <c r="S7" s="389"/>
       <c r="U7" s="314" t="s">
         <v>227</v>
       </c>
       <c r="V7" s="316"/>
     </row>
     <row r="8" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="391" t="s">
+      <c r="A8" s="390" t="s">
         <v>186</v>
       </c>
-      <c r="B8" s="391"/>
-      <c r="C8" s="391"/>
-      <c r="D8" s="391"/>
-      <c r="E8" s="391"/>
-      <c r="F8" s="391"/>
-      <c r="G8" s="391"/>
-      <c r="H8" s="391"/>
-      <c r="I8" s="391"/>
-      <c r="J8" s="391"/>
-      <c r="K8" s="391"/>
-      <c r="L8" s="391"/>
-      <c r="M8" s="391"/>
-      <c r="N8" s="391"/>
-      <c r="O8" s="391"/>
-      <c r="P8" s="391"/>
-      <c r="Q8" s="391"/>
-      <c r="R8" s="391"/>
-      <c r="S8" s="391"/>
+      <c r="B8" s="390"/>
+      <c r="C8" s="390"/>
+      <c r="D8" s="390"/>
+      <c r="E8" s="390"/>
+      <c r="F8" s="390"/>
+      <c r="G8" s="390"/>
+      <c r="H8" s="390"/>
+      <c r="I8" s="390"/>
+      <c r="J8" s="390"/>
+      <c r="K8" s="390"/>
+      <c r="L8" s="390"/>
+      <c r="M8" s="390"/>
+      <c r="N8" s="390"/>
+      <c r="O8" s="390"/>
+      <c r="P8" s="390"/>
+      <c r="Q8" s="390"/>
+      <c r="R8" s="390"/>
+      <c r="S8" s="390"/>
       <c r="U8" s="317"/>
       <c r="V8" s="318"/>
     </row>
@@ -8818,26 +8818,26 @@
       <c r="A10" s="260"/>
       <c r="B10" s="260"/>
       <c r="C10" s="260"/>
-      <c r="D10" s="392" t="s">
+      <c r="D10" s="391" t="s">
         <v>187</v>
       </c>
-      <c r="E10" s="392"/>
-      <c r="F10" s="392"/>
-      <c r="G10" s="392" t="s">
+      <c r="E10" s="391"/>
+      <c r="F10" s="391"/>
+      <c r="G10" s="391" t="s">
         <v>188</v>
       </c>
-      <c r="H10" s="392"/>
-      <c r="I10" s="392"/>
-      <c r="J10" s="392" t="s">
+      <c r="H10" s="391"/>
+      <c r="I10" s="391"/>
+      <c r="J10" s="391" t="s">
         <v>189</v>
       </c>
-      <c r="K10" s="392"/>
-      <c r="L10" s="392"/>
-      <c r="M10" s="355" t="s">
+      <c r="K10" s="391"/>
+      <c r="L10" s="391"/>
+      <c r="M10" s="354" t="s">
         <v>190</v>
       </c>
-      <c r="N10" s="355"/>
-      <c r="O10" s="355"/>
+      <c r="N10" s="354"/>
+      <c r="O10" s="354"/>
       <c r="U10" s="314" t="s">
         <v>59</v>
       </c>
@@ -8847,18 +8847,18 @@
       <c r="A11" s="260"/>
       <c r="B11" s="260"/>
       <c r="C11" s="260"/>
-      <c r="D11" s="393"/>
-      <c r="E11" s="394"/>
-      <c r="F11" s="395"/>
+      <c r="D11" s="392"/>
+      <c r="E11" s="393"/>
+      <c r="F11" s="394"/>
       <c r="G11" s="261"/>
       <c r="H11" s="262"/>
       <c r="I11" s="263"/>
-      <c r="J11" s="393"/>
-      <c r="K11" s="394"/>
-      <c r="L11" s="395"/>
-      <c r="M11" s="396"/>
-      <c r="N11" s="397"/>
-      <c r="O11" s="398"/>
+      <c r="J11" s="392"/>
+      <c r="K11" s="393"/>
+      <c r="L11" s="394"/>
+      <c r="M11" s="395"/>
+      <c r="N11" s="396"/>
+      <c r="O11" s="397"/>
       <c r="U11" s="314" t="s">
         <v>69</v>
       </c>
@@ -8888,54 +8888,54 @@
       <c r="V13" s="318"/>
     </row>
     <row r="14" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="399" t="s">
+      <c r="A14" s="398" t="s">
         <v>191</v>
       </c>
-      <c r="B14" s="400"/>
-      <c r="C14" s="400"/>
-      <c r="D14" s="400"/>
-      <c r="E14" s="400"/>
-      <c r="F14" s="400"/>
-      <c r="G14" s="400"/>
-      <c r="H14" s="400"/>
-      <c r="I14" s="400"/>
-      <c r="J14" s="400"/>
-      <c r="K14" s="400"/>
-      <c r="L14" s="400"/>
-      <c r="M14" s="400"/>
-      <c r="N14" s="400"/>
-      <c r="O14" s="400"/>
-      <c r="P14" s="400"/>
-      <c r="Q14" s="400"/>
-      <c r="R14" s="400"/>
-      <c r="S14" s="401"/>
+      <c r="B14" s="399"/>
+      <c r="C14" s="399"/>
+      <c r="D14" s="399"/>
+      <c r="E14" s="399"/>
+      <c r="F14" s="399"/>
+      <c r="G14" s="399"/>
+      <c r="H14" s="399"/>
+      <c r="I14" s="399"/>
+      <c r="J14" s="399"/>
+      <c r="K14" s="399"/>
+      <c r="L14" s="399"/>
+      <c r="M14" s="399"/>
+      <c r="N14" s="399"/>
+      <c r="O14" s="399"/>
+      <c r="P14" s="399"/>
+      <c r="Q14" s="399"/>
+      <c r="R14" s="399"/>
+      <c r="S14" s="400"/>
       <c r="U14" s="314" t="s">
         <v>55</v>
       </c>
       <c r="V14" s="319"/>
     </row>
     <row r="15" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="402" t="s">
+      <c r="A15" s="401" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="403"/>
-      <c r="C15" s="403"/>
-      <c r="D15" s="403"/>
-      <c r="E15" s="403"/>
-      <c r="F15" s="403"/>
-      <c r="G15" s="403"/>
-      <c r="H15" s="403"/>
-      <c r="I15" s="403"/>
-      <c r="J15" s="403"/>
-      <c r="K15" s="403"/>
-      <c r="L15" s="403"/>
-      <c r="M15" s="403"/>
-      <c r="N15" s="403"/>
-      <c r="O15" s="403"/>
-      <c r="P15" s="403"/>
-      <c r="Q15" s="403"/>
-      <c r="R15" s="403"/>
-      <c r="S15" s="404"/>
+      <c r="B15" s="402"/>
+      <c r="C15" s="402"/>
+      <c r="D15" s="402"/>
+      <c r="E15" s="402"/>
+      <c r="F15" s="402"/>
+      <c r="G15" s="402"/>
+      <c r="H15" s="402"/>
+      <c r="I15" s="402"/>
+      <c r="J15" s="402"/>
+      <c r="K15" s="402"/>
+      <c r="L15" s="402"/>
+      <c r="M15" s="402"/>
+      <c r="N15" s="402"/>
+      <c r="O15" s="402"/>
+      <c r="P15" s="402"/>
+      <c r="Q15" s="402"/>
+      <c r="R15" s="402"/>
+      <c r="S15" s="403"/>
       <c r="U15" s="314" t="s">
         <v>56</v>
       </c>
@@ -8969,16 +8969,16 @@
       <c r="B17" s="268"/>
       <c r="C17" s="268"/>
       <c r="D17" s="268"/>
-      <c r="E17" s="405" t="s">
+      <c r="E17" s="404" t="s">
         <v>36</v>
       </c>
-      <c r="F17" s="406"/>
-      <c r="G17" s="407"/>
-      <c r="I17" s="405" t="s">
+      <c r="F17" s="405"/>
+      <c r="G17" s="406"/>
+      <c r="I17" s="404" t="s">
         <v>192</v>
       </c>
-      <c r="J17" s="406"/>
-      <c r="K17" s="407"/>
+      <c r="J17" s="405"/>
+      <c r="K17" s="406"/>
       <c r="P17" s="268"/>
       <c r="Q17" s="268"/>
       <c r="R17" s="268"/>
@@ -9076,93 +9076,93 @@
       <c r="R20" s="277"/>
     </row>
     <row r="21" spans="1:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="368" t="s">
+      <c r="B21" s="367" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="369"/>
-      <c r="D21" s="372" t="s">
+      <c r="C21" s="368"/>
+      <c r="D21" s="371" t="s">
         <v>198</v>
       </c>
-      <c r="E21" s="373"/>
-      <c r="F21" s="373"/>
-      <c r="G21" s="373"/>
-      <c r="H21" s="374"/>
-      <c r="I21" s="375" t="s">
+      <c r="E21" s="372"/>
+      <c r="F21" s="372"/>
+      <c r="G21" s="372"/>
+      <c r="H21" s="373"/>
+      <c r="I21" s="374" t="s">
         <v>199</v>
       </c>
-      <c r="J21" s="376"/>
-      <c r="K21" s="376"/>
-      <c r="L21" s="377"/>
+      <c r="J21" s="375"/>
+      <c r="K21" s="375"/>
+      <c r="L21" s="376"/>
       <c r="M21" s="280"/>
       <c r="N21" s="269"/>
       <c r="O21" s="281"/>
       <c r="P21" s="282"/>
-      <c r="Q21" s="335"/>
-      <c r="R21" s="335"/>
+      <c r="Q21" s="336"/>
+      <c r="R21" s="336"/>
     </row>
     <row r="22" spans="1:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="370"/>
-      <c r="C22" s="371"/>
-      <c r="D22" s="372" t="s">
+      <c r="B22" s="369"/>
+      <c r="C22" s="370"/>
+      <c r="D22" s="371" t="s">
         <v>200</v>
       </c>
-      <c r="E22" s="373"/>
-      <c r="F22" s="373"/>
-      <c r="G22" s="373"/>
-      <c r="H22" s="374"/>
-      <c r="I22" s="378"/>
-      <c r="J22" s="379"/>
-      <c r="K22" s="379"/>
-      <c r="L22" s="380"/>
+      <c r="E22" s="372"/>
+      <c r="F22" s="372"/>
+      <c r="G22" s="372"/>
+      <c r="H22" s="373"/>
+      <c r="I22" s="377"/>
+      <c r="J22" s="378"/>
+      <c r="K22" s="378"/>
+      <c r="L22" s="379"/>
       <c r="M22" s="280"/>
       <c r="N22" s="269"/>
       <c r="O22" s="283"/>
       <c r="P22" s="284"/>
-      <c r="Q22" s="335"/>
-      <c r="R22" s="335"/>
+      <c r="Q22" s="336"/>
+      <c r="R22" s="336"/>
     </row>
     <row r="23" spans="1:22" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="362" t="s">
+      <c r="B23" s="361" t="s">
         <v>201</v>
       </c>
-      <c r="C23" s="363"/>
-      <c r="D23" s="366" t="s">
+      <c r="C23" s="362"/>
+      <c r="D23" s="365" t="s">
         <v>202</v>
       </c>
-      <c r="E23" s="366"/>
-      <c r="F23" s="366" t="s">
+      <c r="E23" s="365"/>
+      <c r="F23" s="365" t="s">
         <v>4</v>
       </c>
-      <c r="G23" s="366"/>
-      <c r="H23" s="367" t="s">
+      <c r="G23" s="365"/>
+      <c r="H23" s="366" t="s">
         <v>203</v>
       </c>
-      <c r="I23" s="366" t="s">
+      <c r="I23" s="365" t="s">
         <v>204</v>
       </c>
-      <c r="J23" s="366"/>
-      <c r="K23" s="366" t="s">
+      <c r="J23" s="365"/>
+      <c r="K23" s="365" t="s">
         <v>205</v>
       </c>
-      <c r="L23" s="366"/>
+      <c r="L23" s="365"/>
       <c r="N23" s="269"/>
       <c r="O23" s="283"/>
       <c r="P23" s="284"/>
-      <c r="Q23" s="335"/>
-      <c r="R23" s="335"/>
+      <c r="Q23" s="336"/>
+      <c r="R23" s="336"/>
     </row>
     <row r="24" spans="1:22" ht="4.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="364"/>
-      <c r="C24" s="365"/>
-      <c r="D24" s="366"/>
-      <c r="E24" s="366"/>
-      <c r="F24" s="366"/>
-      <c r="G24" s="366"/>
-      <c r="H24" s="367"/>
-      <c r="I24" s="366"/>
-      <c r="J24" s="366"/>
-      <c r="K24" s="366"/>
-      <c r="L24" s="366"/>
+      <c r="B24" s="363"/>
+      <c r="C24" s="364"/>
+      <c r="D24" s="365"/>
+      <c r="E24" s="365"/>
+      <c r="F24" s="365"/>
+      <c r="G24" s="365"/>
+      <c r="H24" s="366"/>
+      <c r="I24" s="365"/>
+      <c r="J24" s="365"/>
+      <c r="K24" s="365"/>
+      <c r="L24" s="365"/>
       <c r="U24" s="286"/>
       <c r="V24" s="286"/>
     </row>
@@ -9173,23 +9173,23 @@
       <c r="C25" s="285" t="s">
         <v>207</v>
       </c>
-      <c r="D25" s="366"/>
-      <c r="E25" s="366"/>
-      <c r="F25" s="366"/>
-      <c r="G25" s="366"/>
-      <c r="H25" s="367"/>
-      <c r="I25" s="366"/>
-      <c r="J25" s="366"/>
-      <c r="K25" s="366"/>
-      <c r="L25" s="366"/>
-      <c r="N25" s="361" t="s">
+      <c r="D25" s="365"/>
+      <c r="E25" s="365"/>
+      <c r="F25" s="365"/>
+      <c r="G25" s="365"/>
+      <c r="H25" s="366"/>
+      <c r="I25" s="365"/>
+      <c r="J25" s="365"/>
+      <c r="K25" s="365"/>
+      <c r="L25" s="365"/>
+      <c r="N25" s="360" t="s">
         <v>37</v>
       </c>
-      <c r="O25" s="361"/>
-      <c r="P25" s="361" t="s">
+      <c r="O25" s="360"/>
+      <c r="P25" s="360" t="s">
         <v>208</v>
       </c>
-      <c r="Q25" s="361"/>
+      <c r="Q25" s="360"/>
       <c r="U25" s="286"/>
       <c r="V25" s="286"/>
     </row>
@@ -9200,25 +9200,25 @@
       <c r="C26" s="288" t="s">
         <v>138</v>
       </c>
-      <c r="D26" s="350"/>
-      <c r="E26" s="351"/>
-      <c r="F26" s="352">
+      <c r="D26" s="351"/>
+      <c r="E26" s="352"/>
+      <c r="F26" s="534">
         <v>4.2454999999999998</v>
       </c>
-      <c r="G26" s="353"/>
+      <c r="G26" s="535"/>
       <c r="H26" s="289"/>
-      <c r="I26" s="350"/>
-      <c r="J26" s="351"/>
-      <c r="K26" s="359"/>
-      <c r="L26" s="360"/>
-      <c r="N26" s="354" t="s">
+      <c r="I26" s="351"/>
+      <c r="J26" s="352"/>
+      <c r="K26" s="358"/>
+      <c r="L26" s="359"/>
+      <c r="N26" s="353" t="s">
         <v>209</v>
       </c>
-      <c r="O26" s="354"/>
-      <c r="P26" s="355">
+      <c r="O26" s="353"/>
+      <c r="P26" s="354">
         <v>20000</v>
       </c>
-      <c r="Q26" s="355"/>
+      <c r="Q26" s="354"/>
       <c r="U26" s="286"/>
       <c r="V26" s="286"/>
     </row>
@@ -9229,25 +9229,25 @@
       <c r="C27" s="288" t="s">
         <v>139</v>
       </c>
-      <c r="D27" s="350"/>
-      <c r="E27" s="351"/>
-      <c r="F27" s="352">
+      <c r="D27" s="351"/>
+      <c r="E27" s="352"/>
+      <c r="F27" s="534">
         <v>18.415600000000001</v>
       </c>
-      <c r="G27" s="353"/>
+      <c r="G27" s="535"/>
       <c r="H27" s="289"/>
-      <c r="I27" s="350"/>
-      <c r="J27" s="351"/>
-      <c r="K27" s="359"/>
-      <c r="L27" s="360"/>
-      <c r="N27" s="354" t="s">
+      <c r="I27" s="351"/>
+      <c r="J27" s="352"/>
+      <c r="K27" s="358"/>
+      <c r="L27" s="359"/>
+      <c r="N27" s="353" t="s">
         <v>138</v>
       </c>
-      <c r="O27" s="354"/>
-      <c r="P27" s="355">
+      <c r="O27" s="353"/>
+      <c r="P27" s="354">
         <v>15000</v>
       </c>
-      <c r="Q27" s="355"/>
+      <c r="Q27" s="354"/>
       <c r="U27" s="286"/>
       <c r="V27" s="286"/>
     </row>
@@ -9258,25 +9258,25 @@
       <c r="C28" s="288" t="s">
         <v>140</v>
       </c>
-      <c r="D28" s="350"/>
-      <c r="E28" s="351"/>
-      <c r="F28" s="352">
+      <c r="D28" s="351"/>
+      <c r="E28" s="352"/>
+      <c r="F28" s="534">
         <v>12.4611</v>
       </c>
-      <c r="G28" s="353"/>
+      <c r="G28" s="535"/>
       <c r="H28" s="289"/>
-      <c r="I28" s="350"/>
-      <c r="J28" s="351"/>
-      <c r="K28" s="359"/>
-      <c r="L28" s="360"/>
-      <c r="N28" s="354" t="s">
+      <c r="I28" s="351"/>
+      <c r="J28" s="352"/>
+      <c r="K28" s="358"/>
+      <c r="L28" s="359"/>
+      <c r="N28" s="353" t="s">
         <v>139</v>
       </c>
-      <c r="O28" s="354"/>
-      <c r="P28" s="355">
+      <c r="O28" s="353"/>
+      <c r="P28" s="354">
         <v>10000</v>
       </c>
-      <c r="Q28" s="355"/>
+      <c r="Q28" s="354"/>
       <c r="U28" s="286"/>
       <c r="V28" s="286"/>
     </row>
@@ -9287,25 +9287,25 @@
       <c r="C29" s="288" t="s">
         <v>141</v>
       </c>
-      <c r="D29" s="350"/>
-      <c r="E29" s="351"/>
-      <c r="F29" s="352">
+      <c r="D29" s="351"/>
+      <c r="E29" s="352"/>
+      <c r="F29" s="534">
         <v>21.021799999999999</v>
       </c>
-      <c r="G29" s="353"/>
+      <c r="G29" s="535"/>
       <c r="H29" s="289"/>
-      <c r="I29" s="350"/>
-      <c r="J29" s="351"/>
-      <c r="K29" s="359"/>
-      <c r="L29" s="360"/>
-      <c r="N29" s="354" t="s">
+      <c r="I29" s="351"/>
+      <c r="J29" s="352"/>
+      <c r="K29" s="358"/>
+      <c r="L29" s="359"/>
+      <c r="N29" s="353" t="s">
         <v>140</v>
       </c>
-      <c r="O29" s="354"/>
-      <c r="P29" s="355">
+      <c r="O29" s="353"/>
+      <c r="P29" s="354">
         <v>5000</v>
       </c>
-      <c r="Q29" s="355"/>
+      <c r="Q29" s="354"/>
     </row>
     <row r="30" spans="1:22" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="288" t="s">
@@ -9314,25 +9314,25 @@
       <c r="C30" s="288" t="s">
         <v>142</v>
       </c>
-      <c r="D30" s="350"/>
-      <c r="E30" s="351"/>
-      <c r="F30" s="352">
+      <c r="D30" s="351"/>
+      <c r="E30" s="352"/>
+      <c r="F30" s="534">
         <v>12.2151</v>
       </c>
-      <c r="G30" s="353"/>
+      <c r="G30" s="535"/>
       <c r="H30" s="289"/>
-      <c r="I30" s="350"/>
-      <c r="J30" s="351"/>
-      <c r="K30" s="359"/>
-      <c r="L30" s="360"/>
-      <c r="N30" s="354" t="s">
+      <c r="I30" s="351"/>
+      <c r="J30" s="352"/>
+      <c r="K30" s="358"/>
+      <c r="L30" s="359"/>
+      <c r="N30" s="353" t="s">
         <v>141</v>
       </c>
-      <c r="O30" s="354"/>
-      <c r="P30" s="355">
+      <c r="O30" s="353"/>
+      <c r="P30" s="354">
         <v>2000</v>
       </c>
-      <c r="Q30" s="355"/>
+      <c r="Q30" s="354"/>
     </row>
     <row r="31" spans="1:22" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="288" t="s">
@@ -9341,50 +9341,50 @@
       <c r="C31" s="288" t="s">
         <v>143</v>
       </c>
-      <c r="D31" s="350"/>
-      <c r="E31" s="351"/>
-      <c r="F31" s="352">
+      <c r="D31" s="351"/>
+      <c r="E31" s="352"/>
+      <c r="F31" s="534">
         <v>31.640899999999998</v>
       </c>
-      <c r="G31" s="353"/>
+      <c r="G31" s="535"/>
       <c r="H31" s="289"/>
-      <c r="I31" s="350"/>
-      <c r="J31" s="351"/>
-      <c r="K31" s="359"/>
-      <c r="L31" s="360"/>
-      <c r="N31" s="354" t="s">
+      <c r="I31" s="351"/>
+      <c r="J31" s="352"/>
+      <c r="K31" s="358"/>
+      <c r="L31" s="359"/>
+      <c r="N31" s="353" t="s">
         <v>142</v>
       </c>
-      <c r="O31" s="354"/>
-      <c r="P31" s="355">
+      <c r="O31" s="353"/>
+      <c r="P31" s="354">
         <v>1000</v>
       </c>
-      <c r="Q31" s="355"/>
-      <c r="V31" s="349"/>
+      <c r="Q31" s="354"/>
+      <c r="V31" s="350"/>
     </row>
     <row r="32" spans="1:22" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="290" t="s">
         <v>6</v>
       </c>
       <c r="C32" s="291"/>
-      <c r="D32" s="350"/>
-      <c r="E32" s="351"/>
-      <c r="F32" s="352">
+      <c r="D32" s="351"/>
+      <c r="E32" s="352"/>
+      <c r="F32" s="534">
         <v>100</v>
       </c>
-      <c r="G32" s="353"/>
+      <c r="G32" s="535"/>
       <c r="H32" s="292"/>
       <c r="I32" s="292"/>
       <c r="J32" s="292"/>
-      <c r="N32" s="354" t="s">
+      <c r="N32" s="353" t="s">
         <v>143</v>
       </c>
-      <c r="O32" s="354"/>
-      <c r="P32" s="355">
+      <c r="O32" s="353"/>
+      <c r="P32" s="354">
         <v>1000</v>
       </c>
-      <c r="Q32" s="355"/>
-      <c r="V32" s="349"/>
+      <c r="Q32" s="354"/>
+      <c r="V32" s="350"/>
     </row>
     <row r="33" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="293" t="s">
@@ -9431,25 +9431,25 @@
     </row>
     <row r="35" spans="1:25" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="295"/>
-      <c r="B35" s="356" t="s">
+      <c r="B35" s="355" t="s">
         <v>193</v>
       </c>
-      <c r="C35" s="357"/>
-      <c r="D35" s="357"/>
-      <c r="E35" s="357"/>
-      <c r="F35" s="357"/>
-      <c r="G35" s="357"/>
-      <c r="H35" s="357"/>
-      <c r="I35" s="357"/>
-      <c r="J35" s="357"/>
-      <c r="K35" s="357"/>
-      <c r="L35" s="357"/>
-      <c r="M35" s="357"/>
-      <c r="N35" s="357"/>
-      <c r="O35" s="357"/>
-      <c r="P35" s="357"/>
-      <c r="Q35" s="357"/>
-      <c r="R35" s="358"/>
+      <c r="C35" s="356"/>
+      <c r="D35" s="356"/>
+      <c r="E35" s="356"/>
+      <c r="F35" s="356"/>
+      <c r="G35" s="356"/>
+      <c r="H35" s="356"/>
+      <c r="I35" s="356"/>
+      <c r="J35" s="356"/>
+      <c r="K35" s="356"/>
+      <c r="L35" s="356"/>
+      <c r="M35" s="356"/>
+      <c r="N35" s="356"/>
+      <c r="O35" s="356"/>
+      <c r="P35" s="356"/>
+      <c r="Q35" s="356"/>
+      <c r="R35" s="357"/>
       <c r="S35" s="295"/>
       <c r="V35" s="298"/>
     </row>
@@ -9464,83 +9464,83 @@
       <c r="H36" s="303"/>
       <c r="I36" s="302"/>
       <c r="J36" s="303"/>
-      <c r="K36" s="340" t="s">
+      <c r="K36" s="341" t="s">
         <v>196</v>
       </c>
-      <c r="L36" s="341"/>
-      <c r="M36" s="341"/>
-      <c r="N36" s="341"/>
-      <c r="O36" s="341"/>
-      <c r="P36" s="341"/>
-      <c r="Q36" s="341"/>
-      <c r="R36" s="342"/>
+      <c r="L36" s="342"/>
+      <c r="M36" s="342"/>
+      <c r="N36" s="342"/>
+      <c r="O36" s="342"/>
+      <c r="P36" s="342"/>
+      <c r="Q36" s="342"/>
+      <c r="R36" s="343"/>
       <c r="S36" s="295"/>
       <c r="U36" s="286"/>
       <c r="V36" s="304"/>
     </row>
     <row r="37" spans="1:25" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="343" t="s">
+      <c r="B37" s="344" t="s">
         <v>207</v>
       </c>
-      <c r="C37" s="345" t="s">
+      <c r="C37" s="346" t="s">
         <v>211</v>
       </c>
-      <c r="D37" s="345"/>
-      <c r="E37" s="345"/>
-      <c r="F37" s="345"/>
-      <c r="G37" s="345" t="s">
+      <c r="D37" s="346"/>
+      <c r="E37" s="346"/>
+      <c r="F37" s="346"/>
+      <c r="G37" s="346" t="s">
         <v>212</v>
       </c>
-      <c r="H37" s="345"/>
-      <c r="I37" s="345"/>
-      <c r="J37" s="345"/>
-      <c r="K37" s="345" t="s">
+      <c r="H37" s="346"/>
+      <c r="I37" s="346"/>
+      <c r="J37" s="346"/>
+      <c r="K37" s="346" t="s">
         <v>213</v>
       </c>
-      <c r="L37" s="345"/>
-      <c r="M37" s="345"/>
-      <c r="N37" s="345"/>
-      <c r="O37" s="345" t="s">
+      <c r="L37" s="346"/>
+      <c r="M37" s="346"/>
+      <c r="N37" s="346"/>
+      <c r="O37" s="346" t="s">
         <v>214</v>
       </c>
-      <c r="P37" s="345"/>
-      <c r="Q37" s="345"/>
-      <c r="R37" s="345"/>
+      <c r="P37" s="346"/>
+      <c r="Q37" s="346"/>
+      <c r="R37" s="346"/>
     </row>
     <row r="38" spans="1:25" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="344"/>
-      <c r="C38" s="346" t="s">
+      <c r="B38" s="345"/>
+      <c r="C38" s="347" t="s">
         <v>215</v>
       </c>
-      <c r="D38" s="346"/>
-      <c r="E38" s="347" t="s">
+      <c r="D38" s="347"/>
+      <c r="E38" s="348" t="s">
         <v>216</v>
       </c>
-      <c r="F38" s="348"/>
-      <c r="G38" s="346" t="s">
+      <c r="F38" s="349"/>
+      <c r="G38" s="347" t="s">
         <v>215</v>
       </c>
-      <c r="H38" s="346"/>
-      <c r="I38" s="346" t="s">
+      <c r="H38" s="347"/>
+      <c r="I38" s="347" t="s">
         <v>216</v>
       </c>
-      <c r="J38" s="346"/>
-      <c r="K38" s="346" t="s">
+      <c r="J38" s="347"/>
+      <c r="K38" s="347" t="s">
         <v>215</v>
       </c>
-      <c r="L38" s="346"/>
-      <c r="M38" s="346" t="s">
+      <c r="L38" s="347"/>
+      <c r="M38" s="347" t="s">
         <v>216</v>
       </c>
-      <c r="N38" s="346"/>
-      <c r="O38" s="346" t="s">
+      <c r="N38" s="347"/>
+      <c r="O38" s="347" t="s">
         <v>215</v>
       </c>
-      <c r="P38" s="346"/>
-      <c r="Q38" s="346" t="s">
+      <c r="P38" s="347"/>
+      <c r="Q38" s="347" t="s">
         <v>216</v>
       </c>
-      <c r="R38" s="346"/>
+      <c r="R38" s="347"/>
       <c r="V38" s="305"/>
       <c r="W38" s="305"/>
       <c r="X38" s="306"/>
@@ -9550,22 +9550,22 @@
       <c r="B39" s="288" t="s">
         <v>138</v>
       </c>
-      <c r="C39" s="336"/>
-      <c r="D39" s="336"/>
-      <c r="E39" s="337"/>
-      <c r="F39" s="337"/>
-      <c r="G39" s="338"/>
-      <c r="H39" s="338"/>
-      <c r="I39" s="337"/>
-      <c r="J39" s="337"/>
-      <c r="K39" s="339"/>
-      <c r="L39" s="339"/>
-      <c r="M39" s="335"/>
-      <c r="N39" s="335"/>
-      <c r="O39" s="335"/>
-      <c r="P39" s="335"/>
-      <c r="Q39" s="335"/>
-      <c r="R39" s="335"/>
+      <c r="C39" s="337"/>
+      <c r="D39" s="337"/>
+      <c r="E39" s="338"/>
+      <c r="F39" s="338"/>
+      <c r="G39" s="339"/>
+      <c r="H39" s="339"/>
+      <c r="I39" s="338"/>
+      <c r="J39" s="338"/>
+      <c r="K39" s="340"/>
+      <c r="L39" s="340"/>
+      <c r="M39" s="336"/>
+      <c r="N39" s="336"/>
+      <c r="O39" s="336"/>
+      <c r="P39" s="336"/>
+      <c r="Q39" s="336"/>
+      <c r="R39" s="336"/>
       <c r="V39" s="298"/>
       <c r="W39" s="298"/>
       <c r="X39" s="305"/>
@@ -9575,22 +9575,22 @@
       <c r="B40" s="288" t="s">
         <v>139</v>
       </c>
-      <c r="C40" s="336"/>
-      <c r="D40" s="336"/>
-      <c r="E40" s="337"/>
-      <c r="F40" s="337"/>
-      <c r="G40" s="338"/>
-      <c r="H40" s="338"/>
-      <c r="I40" s="337"/>
-      <c r="J40" s="337"/>
-      <c r="K40" s="339"/>
-      <c r="L40" s="339"/>
-      <c r="M40" s="335"/>
-      <c r="N40" s="335"/>
-      <c r="O40" s="335"/>
-      <c r="P40" s="335"/>
-      <c r="Q40" s="335"/>
-      <c r="R40" s="335"/>
+      <c r="C40" s="337"/>
+      <c r="D40" s="337"/>
+      <c r="E40" s="338"/>
+      <c r="F40" s="338"/>
+      <c r="G40" s="339"/>
+      <c r="H40" s="339"/>
+      <c r="I40" s="338"/>
+      <c r="J40" s="338"/>
+      <c r="K40" s="340"/>
+      <c r="L40" s="340"/>
+      <c r="M40" s="336"/>
+      <c r="N40" s="336"/>
+      <c r="O40" s="336"/>
+      <c r="P40" s="336"/>
+      <c r="Q40" s="336"/>
+      <c r="R40" s="336"/>
       <c r="V40" s="298"/>
       <c r="W40" s="298"/>
       <c r="X40" s="305"/>
@@ -9600,22 +9600,22 @@
       <c r="B41" s="288" t="s">
         <v>140</v>
       </c>
-      <c r="C41" s="336"/>
-      <c r="D41" s="336"/>
-      <c r="E41" s="337"/>
-      <c r="F41" s="337"/>
-      <c r="G41" s="338"/>
-      <c r="H41" s="338"/>
-      <c r="I41" s="337"/>
-      <c r="J41" s="337"/>
-      <c r="K41" s="339"/>
-      <c r="L41" s="339"/>
-      <c r="M41" s="335"/>
-      <c r="N41" s="335"/>
-      <c r="O41" s="335"/>
-      <c r="P41" s="335"/>
-      <c r="Q41" s="335"/>
-      <c r="R41" s="335"/>
+      <c r="C41" s="337"/>
+      <c r="D41" s="337"/>
+      <c r="E41" s="338"/>
+      <c r="F41" s="338"/>
+      <c r="G41" s="339"/>
+      <c r="H41" s="339"/>
+      <c r="I41" s="338"/>
+      <c r="J41" s="338"/>
+      <c r="K41" s="340"/>
+      <c r="L41" s="340"/>
+      <c r="M41" s="336"/>
+      <c r="N41" s="336"/>
+      <c r="O41" s="336"/>
+      <c r="P41" s="336"/>
+      <c r="Q41" s="336"/>
+      <c r="R41" s="336"/>
       <c r="V41" s="298"/>
       <c r="W41" s="298"/>
       <c r="X41" s="298"/>
@@ -9625,22 +9625,22 @@
       <c r="B42" s="288" t="s">
         <v>141</v>
       </c>
-      <c r="C42" s="336"/>
-      <c r="D42" s="336"/>
-      <c r="E42" s="337"/>
-      <c r="F42" s="337"/>
-      <c r="G42" s="338"/>
-      <c r="H42" s="338"/>
-      <c r="I42" s="337"/>
-      <c r="J42" s="337"/>
-      <c r="K42" s="339"/>
-      <c r="L42" s="339"/>
-      <c r="M42" s="335"/>
-      <c r="N42" s="335"/>
-      <c r="O42" s="335"/>
-      <c r="P42" s="335"/>
-      <c r="Q42" s="335"/>
-      <c r="R42" s="335"/>
+      <c r="C42" s="337"/>
+      <c r="D42" s="337"/>
+      <c r="E42" s="338"/>
+      <c r="F42" s="338"/>
+      <c r="G42" s="339"/>
+      <c r="H42" s="339"/>
+      <c r="I42" s="338"/>
+      <c r="J42" s="338"/>
+      <c r="K42" s="340"/>
+      <c r="L42" s="340"/>
+      <c r="M42" s="336"/>
+      <c r="N42" s="336"/>
+      <c r="O42" s="336"/>
+      <c r="P42" s="336"/>
+      <c r="Q42" s="336"/>
+      <c r="R42" s="336"/>
       <c r="V42" s="298"/>
       <c r="W42" s="298"/>
       <c r="X42" s="298"/>
@@ -9650,22 +9650,22 @@
       <c r="B43" s="288" t="s">
         <v>142</v>
       </c>
-      <c r="C43" s="336"/>
-      <c r="D43" s="336"/>
-      <c r="E43" s="337"/>
-      <c r="F43" s="337"/>
-      <c r="G43" s="338"/>
-      <c r="H43" s="338"/>
-      <c r="I43" s="337"/>
-      <c r="J43" s="337"/>
-      <c r="K43" s="339"/>
-      <c r="L43" s="339"/>
-      <c r="M43" s="335"/>
-      <c r="N43" s="335"/>
-      <c r="O43" s="335"/>
-      <c r="P43" s="335"/>
-      <c r="Q43" s="335"/>
-      <c r="R43" s="335"/>
+      <c r="C43" s="337"/>
+      <c r="D43" s="337"/>
+      <c r="E43" s="338"/>
+      <c r="F43" s="338"/>
+      <c r="G43" s="339"/>
+      <c r="H43" s="339"/>
+      <c r="I43" s="338"/>
+      <c r="J43" s="338"/>
+      <c r="K43" s="340"/>
+      <c r="L43" s="340"/>
+      <c r="M43" s="336"/>
+      <c r="N43" s="336"/>
+      <c r="O43" s="336"/>
+      <c r="P43" s="336"/>
+      <c r="Q43" s="336"/>
+      <c r="R43" s="336"/>
       <c r="V43" s="298"/>
       <c r="W43" s="298"/>
       <c r="X43" s="298"/>
@@ -9675,22 +9675,22 @@
       <c r="B44" s="288" t="s">
         <v>143</v>
       </c>
-      <c r="C44" s="336"/>
-      <c r="D44" s="336"/>
-      <c r="E44" s="337"/>
-      <c r="F44" s="337"/>
-      <c r="G44" s="338"/>
-      <c r="H44" s="338"/>
-      <c r="I44" s="337"/>
-      <c r="J44" s="337"/>
-      <c r="K44" s="339"/>
-      <c r="L44" s="339"/>
-      <c r="M44" s="335"/>
-      <c r="N44" s="335"/>
-      <c r="O44" s="335"/>
-      <c r="P44" s="335"/>
-      <c r="Q44" s="335"/>
-      <c r="R44" s="335"/>
+      <c r="C44" s="337"/>
+      <c r="D44" s="337"/>
+      <c r="E44" s="338"/>
+      <c r="F44" s="338"/>
+      <c r="G44" s="339"/>
+      <c r="H44" s="339"/>
+      <c r="I44" s="338"/>
+      <c r="J44" s="338"/>
+      <c r="K44" s="340"/>
+      <c r="L44" s="340"/>
+      <c r="M44" s="336"/>
+      <c r="N44" s="336"/>
+      <c r="O44" s="336"/>
+      <c r="P44" s="336"/>
+      <c r="Q44" s="336"/>
+      <c r="R44" s="336"/>
       <c r="W44" s="307"/>
       <c r="X44" s="298"/>
       <c r="Y44" s="298"/>
@@ -9712,48 +9712,48 @@
       <c r="Y46" s="298"/>
     </row>
     <row r="47" spans="1:25" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B47" s="329" t="s">
+      <c r="B47" s="330" t="s">
         <v>218</v>
       </c>
-      <c r="C47" s="329"/>
-      <c r="D47" s="330" t="s">
+      <c r="C47" s="330"/>
+      <c r="D47" s="331" t="s">
         <v>219</v>
       </c>
-      <c r="E47" s="330"/>
-      <c r="F47" s="330"/>
-      <c r="G47" s="329"/>
-      <c r="H47" s="329"/>
-      <c r="I47" s="329"/>
-      <c r="J47" s="329"/>
-      <c r="K47" s="331" t="s">
+      <c r="E47" s="331"/>
+      <c r="F47" s="331"/>
+      <c r="G47" s="330"/>
+      <c r="H47" s="330"/>
+      <c r="I47" s="330"/>
+      <c r="J47" s="330"/>
+      <c r="K47" s="332" t="s">
         <v>220</v>
       </c>
-      <c r="L47" s="332"/>
-      <c r="M47" s="333"/>
-      <c r="N47" s="333"/>
-      <c r="O47" s="333"/>
-      <c r="P47" s="333"/>
+      <c r="L47" s="333"/>
+      <c r="M47" s="334"/>
+      <c r="N47" s="334"/>
+      <c r="O47" s="334"/>
+      <c r="P47" s="334"/>
       <c r="X47" s="298"/>
       <c r="Y47" s="298"/>
     </row>
     <row r="48" spans="1:25" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B48" s="329"/>
-      <c r="C48" s="329"/>
-      <c r="D48" s="334" t="s">
+      <c r="B48" s="330"/>
+      <c r="C48" s="330"/>
+      <c r="D48" s="335" t="s">
         <v>221</v>
       </c>
-      <c r="E48" s="334"/>
-      <c r="F48" s="334"/>
-      <c r="G48" s="329"/>
-      <c r="H48" s="329"/>
-      <c r="I48" s="329"/>
-      <c r="J48" s="329"/>
-      <c r="K48" s="331"/>
-      <c r="L48" s="332"/>
-      <c r="M48" s="333"/>
-      <c r="N48" s="333"/>
-      <c r="O48" s="333"/>
-      <c r="P48" s="333"/>
+      <c r="E48" s="335"/>
+      <c r="F48" s="335"/>
+      <c r="G48" s="330"/>
+      <c r="H48" s="330"/>
+      <c r="I48" s="330"/>
+      <c r="J48" s="330"/>
+      <c r="K48" s="332"/>
+      <c r="L48" s="333"/>
+      <c r="M48" s="334"/>
+      <c r="N48" s="334"/>
+      <c r="O48" s="334"/>
+      <c r="P48" s="334"/>
       <c r="X48" s="298"/>
       <c r="Y48" s="298"/>
     </row>
@@ -9825,27 +9825,27 @@
     </row>
     <row r="55" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="56" spans="1:25" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="328" t="s">
+      <c r="A56" s="329" t="s">
         <v>223</v>
       </c>
-      <c r="B56" s="328"/>
-      <c r="C56" s="328"/>
-      <c r="D56" s="328"/>
-      <c r="E56" s="328"/>
-      <c r="F56" s="328"/>
-      <c r="G56" s="328"/>
-      <c r="H56" s="328"/>
-      <c r="I56" s="328"/>
-      <c r="J56" s="328"/>
-      <c r="K56" s="328"/>
-      <c r="L56" s="328"/>
-      <c r="M56" s="328"/>
-      <c r="N56" s="328"/>
-      <c r="O56" s="328"/>
-      <c r="P56" s="328"/>
-      <c r="Q56" s="328"/>
-      <c r="R56" s="328"/>
-      <c r="S56" s="328"/>
+      <c r="B56" s="329"/>
+      <c r="C56" s="329"/>
+      <c r="D56" s="329"/>
+      <c r="E56" s="329"/>
+      <c r="F56" s="329"/>
+      <c r="G56" s="329"/>
+      <c r="H56" s="329"/>
+      <c r="I56" s="329"/>
+      <c r="J56" s="329"/>
+      <c r="K56" s="329"/>
+      <c r="L56" s="329"/>
+      <c r="M56" s="329"/>
+      <c r="N56" s="329"/>
+      <c r="O56" s="329"/>
+      <c r="P56" s="329"/>
+      <c r="Q56" s="329"/>
+      <c r="R56" s="329"/>
+      <c r="S56" s="329"/>
     </row>
   </sheetData>
   <protectedRanges>
@@ -10039,40 +10039,40 @@
       <c r="N1" s="39"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="443" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="443"/>
-      <c r="C2" s="443"/>
-      <c r="D2" s="443"/>
-      <c r="E2" s="443"/>
-      <c r="F2" s="443"/>
-      <c r="G2" s="443"/>
-      <c r="H2" s="443"/>
-      <c r="I2" s="443"/>
-      <c r="J2" s="443"/>
-      <c r="K2" s="443"/>
-      <c r="L2" s="443"/>
-      <c r="M2" s="443"/>
-      <c r="N2" s="443"/>
+      <c r="A2" s="442" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="442"/>
+      <c r="C2" s="442"/>
+      <c r="D2" s="442"/>
+      <c r="E2" s="442"/>
+      <c r="F2" s="442"/>
+      <c r="G2" s="442"/>
+      <c r="H2" s="442"/>
+      <c r="I2" s="442"/>
+      <c r="J2" s="442"/>
+      <c r="K2" s="442"/>
+      <c r="L2" s="442"/>
+      <c r="M2" s="442"/>
+      <c r="N2" s="442"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="444">
+      <c r="A3" s="443">
         <v>1</v>
       </c>
-      <c r="B3" s="444"/>
-      <c r="C3" s="444"/>
-      <c r="D3" s="444"/>
-      <c r="E3" s="444"/>
-      <c r="F3" s="444"/>
-      <c r="G3" s="444"/>
-      <c r="H3" s="444"/>
-      <c r="I3" s="444"/>
-      <c r="J3" s="444"/>
-      <c r="K3" s="444"/>
-      <c r="L3" s="444"/>
-      <c r="M3" s="444"/>
-      <c r="N3" s="444"/>
+      <c r="B3" s="443"/>
+      <c r="C3" s="443"/>
+      <c r="D3" s="443"/>
+      <c r="E3" s="443"/>
+      <c r="F3" s="443"/>
+      <c r="G3" s="443"/>
+      <c r="H3" s="443"/>
+      <c r="I3" s="443"/>
+      <c r="J3" s="443"/>
+      <c r="K3" s="443"/>
+      <c r="L3" s="443"/>
+      <c r="M3" s="443"/>
+      <c r="N3" s="443"/>
     </row>
     <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="63"/>
@@ -10097,17 +10097,17 @@
       <c r="B5" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="451">
+      <c r="C5" s="450">
         <f>+FORMATO!V4</f>
         <v>0</v>
       </c>
-      <c r="D5" s="451"/>
-      <c r="E5" s="451"/>
-      <c r="F5" s="451"/>
-      <c r="G5" s="451"/>
-      <c r="H5" s="451"/>
-      <c r="I5" s="451"/>
-      <c r="J5" s="451"/>
+      <c r="D5" s="450"/>
+      <c r="E5" s="450"/>
+      <c r="F5" s="450"/>
+      <c r="G5" s="450"/>
+      <c r="H5" s="450"/>
+      <c r="I5" s="450"/>
+      <c r="J5" s="450"/>
       <c r="K5" s="9" t="s">
         <v>57</v>
       </c>
@@ -10125,17 +10125,17 @@
       <c r="B6" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C6" s="451">
+      <c r="C6" s="450">
         <f>+FORMATO!V5</f>
         <v>0</v>
       </c>
-      <c r="D6" s="451"/>
-      <c r="E6" s="451"/>
-      <c r="F6" s="451"/>
-      <c r="G6" s="451"/>
-      <c r="H6" s="451"/>
-      <c r="I6" s="451"/>
-      <c r="J6" s="451"/>
+      <c r="D6" s="450"/>
+      <c r="E6" s="450"/>
+      <c r="F6" s="450"/>
+      <c r="G6" s="450"/>
+      <c r="H6" s="450"/>
+      <c r="I6" s="450"/>
+      <c r="J6" s="450"/>
       <c r="K6" s="322" t="s">
         <v>58</v>
       </c>
@@ -10154,17 +10154,17 @@
       <c r="B7" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C7" s="451">
+      <c r="C7" s="450">
         <f>+FORMATO!V6</f>
         <v>0</v>
       </c>
-      <c r="D7" s="451"/>
-      <c r="E7" s="451"/>
-      <c r="F7" s="451"/>
-      <c r="G7" s="451"/>
-      <c r="H7" s="451"/>
-      <c r="I7" s="451"/>
-      <c r="J7" s="451"/>
+      <c r="D7" s="450"/>
+      <c r="E7" s="450"/>
+      <c r="F7" s="450"/>
+      <c r="G7" s="450"/>
+      <c r="H7" s="450"/>
+      <c r="I7" s="450"/>
+      <c r="J7" s="450"/>
       <c r="K7" s="10" t="s">
         <v>69</v>
       </c>
@@ -10184,17 +10184,17 @@
       <c r="B8" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="451">
+      <c r="C8" s="450">
         <f>+FORMATO!V7</f>
         <v>0</v>
       </c>
-      <c r="D8" s="451"/>
-      <c r="E8" s="451"/>
-      <c r="F8" s="451"/>
-      <c r="G8" s="451"/>
-      <c r="H8" s="451"/>
-      <c r="I8" s="451"/>
-      <c r="J8" s="451"/>
+      <c r="D8" s="450"/>
+      <c r="E8" s="450"/>
+      <c r="F8" s="450"/>
+      <c r="G8" s="450"/>
+      <c r="H8" s="450"/>
+      <c r="I8" s="450"/>
+      <c r="J8" s="450"/>
       <c r="K8" s="10" t="s">
         <v>59</v>
       </c>
@@ -10226,40 +10226,40 @@
       <c r="N9" s="39"/>
     </row>
     <row r="10" spans="1:14" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="445" t="s">
+      <c r="A10" s="444" t="s">
         <v>27</v>
       </c>
-      <c r="B10" s="446"/>
-      <c r="C10" s="446"/>
-      <c r="D10" s="446"/>
-      <c r="E10" s="446"/>
-      <c r="F10" s="446"/>
-      <c r="G10" s="446"/>
-      <c r="H10" s="446"/>
-      <c r="I10" s="446"/>
-      <c r="J10" s="446"/>
-      <c r="K10" s="446"/>
-      <c r="L10" s="446"/>
-      <c r="M10" s="446"/>
-      <c r="N10" s="447"/>
+      <c r="B10" s="445"/>
+      <c r="C10" s="445"/>
+      <c r="D10" s="445"/>
+      <c r="E10" s="445"/>
+      <c r="F10" s="445"/>
+      <c r="G10" s="445"/>
+      <c r="H10" s="445"/>
+      <c r="I10" s="445"/>
+      <c r="J10" s="445"/>
+      <c r="K10" s="445"/>
+      <c r="L10" s="445"/>
+      <c r="M10" s="445"/>
+      <c r="N10" s="446"/>
     </row>
     <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="448" t="s">
+      <c r="A11" s="447" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="449"/>
-      <c r="C11" s="449"/>
-      <c r="D11" s="449"/>
-      <c r="E11" s="449"/>
-      <c r="F11" s="449"/>
-      <c r="G11" s="449"/>
-      <c r="H11" s="449"/>
-      <c r="I11" s="449"/>
-      <c r="J11" s="449"/>
-      <c r="K11" s="449"/>
-      <c r="L11" s="449"/>
-      <c r="M11" s="449"/>
-      <c r="N11" s="450"/>
+      <c r="B11" s="448"/>
+      <c r="C11" s="448"/>
+      <c r="D11" s="448"/>
+      <c r="E11" s="448"/>
+      <c r="F11" s="448"/>
+      <c r="G11" s="448"/>
+      <c r="H11" s="448"/>
+      <c r="I11" s="448"/>
+      <c r="J11" s="448"/>
+      <c r="K11" s="448"/>
+      <c r="L11" s="448"/>
+      <c r="M11" s="448"/>
+      <c r="N11" s="449"/>
     </row>
     <row r="12" spans="1:14" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="54"/>
@@ -10278,15 +10278,15 @@
       <c r="N12" s="44"/>
     </row>
     <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="439" t="s">
+      <c r="A13" s="438" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="440"/>
-      <c r="C13" s="440"/>
-      <c r="D13" s="440"/>
-      <c r="E13" s="440"/>
-      <c r="F13" s="440"/>
-      <c r="G13" s="440"/>
+      <c r="B13" s="439"/>
+      <c r="C13" s="439"/>
+      <c r="D13" s="439"/>
+      <c r="E13" s="439"/>
+      <c r="F13" s="439"/>
+      <c r="G13" s="439"/>
       <c r="H13" s="39"/>
       <c r="I13" s="39"/>
       <c r="J13" s="39"/>
@@ -10319,11 +10319,11 @@
       <c r="L14" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="M14" s="441">
+      <c r="M14" s="440">
         <f>+FORMATO!V13</f>
         <v>0</v>
       </c>
-      <c r="N14" s="442"/>
+      <c r="N14" s="441"/>
     </row>
     <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
@@ -10427,114 +10427,114 @@
       <c r="O18" s="14"/>
     </row>
     <row r="19" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="433" t="s">
+      <c r="A19" s="432" t="s">
         <v>63</v>
       </c>
-      <c r="B19" s="412" t="s">
+      <c r="B19" s="411" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="413"/>
-      <c r="D19" s="414"/>
-      <c r="E19" s="428" t="s">
+      <c r="C19" s="412"/>
+      <c r="D19" s="413"/>
+      <c r="E19" s="427" t="s">
         <v>68</v>
       </c>
-      <c r="F19" s="413" t="s">
+      <c r="F19" s="412" t="s">
         <v>174</v>
       </c>
-      <c r="G19" s="414"/>
-      <c r="H19" s="412" t="s">
+      <c r="G19" s="413"/>
+      <c r="H19" s="411" t="s">
         <v>175</v>
       </c>
-      <c r="I19" s="414"/>
-      <c r="J19" s="412" t="s">
+      <c r="I19" s="413"/>
+      <c r="J19" s="411" t="s">
         <v>176</v>
       </c>
-      <c r="K19" s="414"/>
-      <c r="L19" s="412" t="s">
+      <c r="K19" s="413"/>
+      <c r="L19" s="411" t="s">
         <v>177</v>
       </c>
-      <c r="M19" s="413"/>
-      <c r="N19" s="414"/>
+      <c r="M19" s="412"/>
+      <c r="N19" s="413"/>
       <c r="O19" s="15"/>
     </row>
     <row r="20" spans="1:17" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="434"/>
-      <c r="B20" s="422"/>
-      <c r="C20" s="423"/>
-      <c r="D20" s="424"/>
-      <c r="E20" s="429"/>
-      <c r="F20" s="416"/>
-      <c r="G20" s="417"/>
-      <c r="H20" s="415"/>
-      <c r="I20" s="417"/>
-      <c r="J20" s="415"/>
-      <c r="K20" s="417"/>
-      <c r="L20" s="415"/>
-      <c r="M20" s="416"/>
-      <c r="N20" s="417"/>
+      <c r="A20" s="433"/>
+      <c r="B20" s="421"/>
+      <c r="C20" s="422"/>
+      <c r="D20" s="423"/>
+      <c r="E20" s="428"/>
+      <c r="F20" s="415"/>
+      <c r="G20" s="416"/>
+      <c r="H20" s="414"/>
+      <c r="I20" s="416"/>
+      <c r="J20" s="414"/>
+      <c r="K20" s="416"/>
+      <c r="L20" s="414"/>
+      <c r="M20" s="415"/>
+      <c r="N20" s="416"/>
     </row>
     <row r="21" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="434"/>
-      <c r="B21" s="415"/>
-      <c r="C21" s="416"/>
-      <c r="D21" s="417"/>
-      <c r="E21" s="430"/>
-      <c r="F21" s="419" t="s">
+      <c r="A21" s="433"/>
+      <c r="B21" s="414"/>
+      <c r="C21" s="415"/>
+      <c r="D21" s="416"/>
+      <c r="E21" s="429"/>
+      <c r="F21" s="418" t="s">
         <v>26</v>
       </c>
-      <c r="G21" s="431" t="s">
+      <c r="G21" s="430" t="s">
         <v>48</v>
       </c>
-      <c r="H21" s="431" t="s">
+      <c r="H21" s="430" t="s">
         <v>26</v>
       </c>
-      <c r="I21" s="431" t="s">
+      <c r="I21" s="430" t="s">
         <v>48</v>
       </c>
-      <c r="J21" s="431" t="s">
+      <c r="J21" s="430" t="s">
         <v>26</v>
       </c>
-      <c r="K21" s="431" t="s">
+      <c r="K21" s="430" t="s">
         <v>48</v>
       </c>
-      <c r="L21" s="418" t="s">
+      <c r="L21" s="417" t="s">
         <v>26</v>
       </c>
-      <c r="M21" s="419"/>
-      <c r="N21" s="431" t="s">
+      <c r="M21" s="418"/>
+      <c r="N21" s="430" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="435"/>
-      <c r="B22" s="425" t="s">
+      <c r="A22" s="434"/>
+      <c r="B22" s="424" t="s">
         <v>4</v>
       </c>
-      <c r="C22" s="426"/>
-      <c r="D22" s="427"/>
+      <c r="C22" s="425"/>
+      <c r="D22" s="426"/>
       <c r="E22" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="432"/>
-      <c r="G22" s="432"/>
-      <c r="H22" s="432"/>
-      <c r="I22" s="432"/>
-      <c r="J22" s="432"/>
-      <c r="K22" s="432"/>
-      <c r="L22" s="420"/>
-      <c r="M22" s="421"/>
-      <c r="N22" s="432"/>
+      <c r="F22" s="431"/>
+      <c r="G22" s="431"/>
+      <c r="H22" s="431"/>
+      <c r="I22" s="431"/>
+      <c r="J22" s="431"/>
+      <c r="K22" s="431"/>
+      <c r="L22" s="419"/>
+      <c r="M22" s="420"/>
+      <c r="N22" s="431"/>
     </row>
     <row r="23" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="B23" s="409" t="e">
+      <c r="B23" s="408" t="e">
         <f>+IF(DATOS!E12=0,"--",DATOS!E12)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C23" s="409"/>
-      <c r="D23" s="409"/>
+      <c r="C23" s="408"/>
+      <c r="D23" s="408"/>
       <c r="E23" s="69" t="e">
         <f>IF(DATOS!E12=0,"--",DATOS!F12)</f>
         <v>#DIV/0!</v>
@@ -10563,11 +10563,11 @@
         <f>+IF(DATOS!G12=0,"--",IF(DATOS!E12&lt;10,"--",DATOS!X12/DATOS!E12/100))</f>
         <v>--</v>
       </c>
-      <c r="L23" s="410" t="str">
+      <c r="L23" s="409" t="str">
         <f>+IF(DATOS!G12=0,"--",IF(DATOS!E12&lt;10,"--",(DATOS!AA12/DATOS!H12)*100))</f>
         <v>--</v>
       </c>
-      <c r="M23" s="411"/>
+      <c r="M23" s="410"/>
       <c r="N23" s="70" t="str">
         <f>+IF(DATOS!G12=0,"--",DATOS!AB12*DATOS!E12/100)</f>
         <v>--</v>
@@ -10578,12 +10578,12 @@
       <c r="A24" s="37" t="s">
         <v>139</v>
       </c>
-      <c r="B24" s="409" t="e">
+      <c r="B24" s="408" t="e">
         <f>+IF(DATOS!E13=0,"--",DATOS!E13)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C24" s="409"/>
-      <c r="D24" s="409"/>
+      <c r="C24" s="408"/>
+      <c r="D24" s="408"/>
       <c r="E24" s="69" t="e">
         <f>IF(DATOS!E13=0,"--",DATOS!F13)</f>
         <v>#DIV/0!</v>
@@ -10612,11 +10612,11 @@
         <f>+IF(DATOS!G13=0,"--",IF(DATOS!E13&lt;10,"--",DATOS!X13/DATOS!E13/100))</f>
         <v>--</v>
       </c>
-      <c r="L24" s="410" t="str">
+      <c r="L24" s="409" t="str">
         <f>+IF(DATOS!G13=0,"--",IF(DATOS!E13&lt;10,"--",(DATOS!AA13/DATOS!H13)*100))</f>
         <v>--</v>
       </c>
-      <c r="M24" s="411"/>
+      <c r="M24" s="410"/>
       <c r="N24" s="70" t="str">
         <f>+IF(DATOS!G13=0,"--",DATOS!AB13*DATOS!E13/100)</f>
         <v>--</v>
@@ -10627,12 +10627,12 @@
       <c r="A25" s="37" t="s">
         <v>140</v>
       </c>
-      <c r="B25" s="409" t="e">
+      <c r="B25" s="408" t="e">
         <f>+IF(DATOS!E14=0,"--",DATOS!E14)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C25" s="409"/>
-      <c r="D25" s="409"/>
+      <c r="C25" s="408"/>
+      <c r="D25" s="408"/>
       <c r="E25" s="69" t="e">
         <f>IF(DATOS!E14=0,"--",DATOS!F14)</f>
         <v>#DIV/0!</v>
@@ -10661,11 +10661,11 @@
         <f>+IF(DATOS!G14=0,"--",IF(DATOS!E14&lt;10,"--",DATOS!X14/DATOS!E14/100))</f>
         <v>--</v>
       </c>
-      <c r="L25" s="410" t="str">
+      <c r="L25" s="409" t="str">
         <f>+IF(DATOS!G14=0,"--",IF(DATOS!E14&lt;10,"--",(DATOS!AA14/DATOS!H14)*100))</f>
         <v>--</v>
       </c>
-      <c r="M25" s="411"/>
+      <c r="M25" s="410"/>
       <c r="N25" s="70" t="str">
         <f>+IF(DATOS!G14=0,"--",DATOS!AB14*DATOS!E14/100)</f>
         <v>--</v>
@@ -10676,12 +10676,12 @@
       <c r="A26" s="37" t="s">
         <v>141</v>
       </c>
-      <c r="B26" s="409" t="e">
+      <c r="B26" s="408" t="e">
         <f>+IF(DATOS!E15=0,"--",DATOS!E15)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C26" s="409"/>
-      <c r="D26" s="409"/>
+      <c r="C26" s="408"/>
+      <c r="D26" s="408"/>
       <c r="E26" s="69" t="e">
         <f>IF(DATOS!E15=0,"--",DATOS!F15)</f>
         <v>#DIV/0!</v>
@@ -10710,11 +10710,11 @@
         <f>+IF(DATOS!G15=0,"--",IF(DATOS!E15&lt;10,"--",DATOS!X15/DATOS!E15/100))</f>
         <v>--</v>
       </c>
-      <c r="L26" s="410" t="str">
+      <c r="L26" s="409" t="str">
         <f>+IF(DATOS!G15=0,"--",IF(DATOS!E15&lt;10,"--",(DATOS!AA15/DATOS!H15)*100))</f>
         <v>--</v>
       </c>
-      <c r="M26" s="411"/>
+      <c r="M26" s="410"/>
       <c r="N26" s="70" t="str">
         <f>+IF(DATOS!G15=0,"--",DATOS!AB15*DATOS!E15/100)</f>
         <v>--</v>
@@ -10725,12 +10725,12 @@
       <c r="A27" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="B27" s="409" t="e">
+      <c r="B27" s="408" t="e">
         <f>+IF(DATOS!E16=0,"--",DATOS!E16)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C27" s="409"/>
-      <c r="D27" s="409"/>
+      <c r="C27" s="408"/>
+      <c r="D27" s="408"/>
       <c r="E27" s="69" t="e">
         <f>IF(DATOS!E16=0,"--",DATOS!F16)</f>
         <v>#DIV/0!</v>
@@ -10759,11 +10759,11 @@
         <f>+IF(DATOS!G16=0,"--",IF(DATOS!E16&lt;10,"--",DATOS!X16/DATOS!E16/100))</f>
         <v>--</v>
       </c>
-      <c r="L27" s="410" t="str">
+      <c r="L27" s="409" t="str">
         <f>+IF(DATOS!G16=0,"--",IF(DATOS!E16&lt;10,"--",(DATOS!AA16/DATOS!H16)*100))</f>
         <v>--</v>
       </c>
-      <c r="M27" s="411"/>
+      <c r="M27" s="410"/>
       <c r="N27" s="70" t="str">
         <f>+IF(DATOS!G16=0,"--",DATOS!AB16*DATOS!E16/100)</f>
         <v>--</v>
@@ -10774,12 +10774,12 @@
       <c r="A28" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="B28" s="409" t="e">
+      <c r="B28" s="408" t="e">
         <f>+IF(DATOS!E17=0,"--",DATOS!E17)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C28" s="409"/>
-      <c r="D28" s="409"/>
+      <c r="C28" s="408"/>
+      <c r="D28" s="408"/>
       <c r="E28" s="69" t="e">
         <f>IF(DATOS!E17=0,"--",DATOS!F17)</f>
         <v>#DIV/0!</v>
@@ -10808,11 +10808,11 @@
         <f>+IF(DATOS!G17=0,"--",IF(DATOS!E17&lt;10,"--",DATOS!X17/DATOS!E17/100))</f>
         <v>--</v>
       </c>
-      <c r="L28" s="410" t="str">
+      <c r="L28" s="409" t="str">
         <f>+IF(DATOS!G17=0,"--",IF(DATOS!E17&lt;10,"--",(DATOS!AA17/DATOS!H17)*100))</f>
         <v>--</v>
       </c>
-      <c r="M28" s="411"/>
+      <c r="M28" s="410"/>
       <c r="N28" s="70" t="str">
         <f>+IF(DATOS!G17=0,"--",DATOS!AB17*DATOS!E17/100)</f>
         <v>--</v>
@@ -10823,12 +10823,12 @@
       <c r="A29" s="180" t="s">
         <v>6</v>
       </c>
-      <c r="B29" s="438" t="e">
+      <c r="B29" s="437" t="e">
         <f>+DATOS!E18</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="C29" s="438"/>
-      <c r="D29" s="438"/>
+      <c r="C29" s="437"/>
+      <c r="D29" s="437"/>
       <c r="E29" s="72"/>
       <c r="F29" s="20"/>
       <c r="G29" s="73">
@@ -10879,11 +10879,11 @@
       <c r="D31" s="21"/>
       <c r="E31" s="21"/>
       <c r="F31" s="21"/>
-      <c r="G31" s="436" t="str">
+      <c r="G31" s="435" t="str">
         <f>+DATOS!F3</f>
         <v>-</v>
       </c>
-      <c r="H31" s="437"/>
+      <c r="H31" s="436"/>
       <c r="I31" s="75"/>
       <c r="J31" s="21"/>
       <c r="K31" s="21"/>
@@ -10900,11 +10900,11 @@
       <c r="D32" s="21"/>
       <c r="E32" s="21"/>
       <c r="F32" s="21"/>
-      <c r="G32" s="436" t="str">
+      <c r="G32" s="435" t="str">
         <f>+DATOS!F5</f>
         <v>-</v>
       </c>
-      <c r="H32" s="437"/>
+      <c r="H32" s="436"/>
       <c r="I32" s="21"/>
       <c r="J32" s="21"/>
       <c r="K32" s="21"/>
@@ -10921,11 +10921,11 @@
       <c r="D33" s="21"/>
       <c r="E33" s="21"/>
       <c r="F33" s="21"/>
-      <c r="G33" s="436">
+      <c r="G33" s="435">
         <f>100-N29</f>
         <v>100</v>
       </c>
-      <c r="H33" s="437"/>
+      <c r="H33" s="436"/>
       <c r="I33" s="21"/>
       <c r="J33" s="21"/>
       <c r="K33" s="21"/>
@@ -11004,22 +11004,22 @@
       <c r="N37" s="18"/>
     </row>
     <row r="38" spans="1:15" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="408" t="s">
+      <c r="A38" s="407" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="408"/>
-      <c r="C38" s="408"/>
-      <c r="D38" s="408"/>
-      <c r="E38" s="408"/>
-      <c r="F38" s="408"/>
-      <c r="G38" s="408"/>
-      <c r="H38" s="408"/>
-      <c r="I38" s="408"/>
-      <c r="J38" s="408"/>
-      <c r="K38" s="408"/>
-      <c r="L38" s="408"/>
-      <c r="M38" s="408"/>
-      <c r="N38" s="408"/>
+      <c r="B38" s="407"/>
+      <c r="C38" s="407"/>
+      <c r="D38" s="407"/>
+      <c r="E38" s="407"/>
+      <c r="F38" s="407"/>
+      <c r="G38" s="407"/>
+      <c r="H38" s="407"/>
+      <c r="I38" s="407"/>
+      <c r="J38" s="407"/>
+      <c r="K38" s="407"/>
+      <c r="L38" s="407"/>
+      <c r="M38" s="407"/>
+      <c r="N38" s="407"/>
     </row>
     <row r="39" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="26" t="s">
@@ -11040,22 +11040,22 @@
       <c r="N39" s="18"/>
     </row>
     <row r="40" spans="1:15" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="408" t="s">
+      <c r="A40" s="407" t="s">
         <v>180</v>
       </c>
-      <c r="B40" s="408"/>
-      <c r="C40" s="408"/>
-      <c r="D40" s="408"/>
-      <c r="E40" s="408"/>
-      <c r="F40" s="408"/>
-      <c r="G40" s="408"/>
-      <c r="H40" s="408"/>
-      <c r="I40" s="408"/>
-      <c r="J40" s="408"/>
-      <c r="K40" s="408"/>
-      <c r="L40" s="408"/>
-      <c r="M40" s="408"/>
-      <c r="N40" s="408"/>
+      <c r="B40" s="407"/>
+      <c r="C40" s="407"/>
+      <c r="D40" s="407"/>
+      <c r="E40" s="407"/>
+      <c r="F40" s="407"/>
+      <c r="G40" s="407"/>
+      <c r="H40" s="407"/>
+      <c r="I40" s="407"/>
+      <c r="J40" s="407"/>
+      <c r="K40" s="407"/>
+      <c r="L40" s="407"/>
+      <c r="M40" s="407"/>
+      <c r="N40" s="407"/>
     </row>
     <row r="41" spans="1:15" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="27"/>
@@ -11363,40 +11363,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.25">
-      <c r="B1" s="483" t="s">
+      <c r="B1" s="482" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="483"/>
-      <c r="D1" s="483"/>
-      <c r="E1" s="483"/>
-      <c r="F1" s="483"/>
-      <c r="G1" s="483"/>
-      <c r="H1" s="483"/>
-      <c r="I1" s="483"/>
-      <c r="J1" s="483"/>
-      <c r="K1" s="483"/>
-      <c r="L1" s="483"/>
-      <c r="M1" s="483"/>
-      <c r="N1" s="483"/>
-      <c r="O1" s="483"/>
-      <c r="P1" s="483"/>
-      <c r="Q1" s="483"/>
-      <c r="R1" s="483"/>
-      <c r="S1" s="483"/>
-      <c r="T1" s="483"/>
-      <c r="U1" s="483"/>
-      <c r="V1" s="483"/>
-      <c r="W1" s="483"/>
-      <c r="X1" s="483"/>
-      <c r="Y1" s="483"/>
-      <c r="Z1" s="483"/>
-      <c r="AA1" s="483"/>
-      <c r="AB1" s="483"/>
-      <c r="AC1" s="483"/>
+      <c r="C1" s="482"/>
+      <c r="D1" s="482"/>
+      <c r="E1" s="482"/>
+      <c r="F1" s="482"/>
+      <c r="G1" s="482"/>
+      <c r="H1" s="482"/>
+      <c r="I1" s="482"/>
+      <c r="J1" s="482"/>
+      <c r="K1" s="482"/>
+      <c r="L1" s="482"/>
+      <c r="M1" s="482"/>
+      <c r="N1" s="482"/>
+      <c r="O1" s="482"/>
+      <c r="P1" s="482"/>
+      <c r="Q1" s="482"/>
+      <c r="R1" s="482"/>
+      <c r="S1" s="482"/>
+      <c r="T1" s="482"/>
+      <c r="U1" s="482"/>
+      <c r="V1" s="482"/>
+      <c r="W1" s="482"/>
+      <c r="X1" s="482"/>
+      <c r="Y1" s="482"/>
+      <c r="Z1" s="482"/>
+      <c r="AA1" s="482"/>
+      <c r="AB1" s="482"/>
+      <c r="AC1" s="482"/>
     </row>
     <row r="2" spans="1:29" ht="5.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F2" s="482"/>
-      <c r="G2" s="482"/>
+      <c r="F2" s="481"/>
+      <c r="G2" s="481"/>
     </row>
     <row r="3" spans="1:29" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="139" t="s">
@@ -11405,10 +11405,10 @@
       <c r="C3" s="171"/>
       <c r="D3" s="140"/>
       <c r="E3" s="141"/>
-      <c r="F3" s="475" t="s">
+      <c r="F3" s="474" t="s">
         <v>179</v>
       </c>
-      <c r="G3" s="476"/>
+      <c r="G3" s="475"/>
       <c r="I3" s="138" t="s">
         <v>120</v>
       </c>
@@ -11429,10 +11429,10 @@
       <c r="C4" s="140"/>
       <c r="D4" s="140"/>
       <c r="E4" s="141"/>
-      <c r="F4" s="477" t="s">
+      <c r="F4" s="476" t="s">
         <v>179</v>
       </c>
-      <c r="G4" s="478"/>
+      <c r="G4" s="477"/>
       <c r="I4" s="138" t="s">
         <v>121</v>
       </c>
@@ -11443,26 +11443,26 @@
       <c r="M4" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="N4" s="452" t="s">
+      <c r="N4" s="451" t="s">
         <v>40</v>
       </c>
-      <c r="O4" s="492"/>
-      <c r="P4" s="452" t="s">
+      <c r="O4" s="491"/>
+      <c r="P4" s="451" t="s">
         <v>70</v>
       </c>
-      <c r="Q4" s="453"/>
-      <c r="R4" s="491" t="s">
+      <c r="Q4" s="452"/>
+      <c r="R4" s="490" t="s">
         <v>71</v>
       </c>
-      <c r="S4" s="491"/>
-      <c r="U4" s="495" t="s">
+      <c r="S4" s="490"/>
+      <c r="U4" s="494" t="s">
         <v>72</v>
       </c>
-      <c r="V4" s="495"/>
-      <c r="W4" s="496" t="s">
+      <c r="V4" s="494"/>
+      <c r="W4" s="495" t="s">
         <v>179</v>
       </c>
-      <c r="X4" s="497"/>
+      <c r="X4" s="496"/>
       <c r="Y4" s="35">
         <f>+FORMATO!M11</f>
         <v>0</v>
@@ -11476,10 +11476,10 @@
       <c r="C5" s="140"/>
       <c r="D5" s="140"/>
       <c r="E5" s="141"/>
-      <c r="F5" s="479" t="s">
+      <c r="F5" s="478" t="s">
         <v>179</v>
       </c>
-      <c r="G5" s="480"/>
+      <c r="G5" s="479"/>
       <c r="H5" s="61"/>
       <c r="I5" s="134" t="s">
         <v>122</v>
@@ -11491,21 +11491,21 @@
       <c r="M5" s="62">
         <v>1</v>
       </c>
-      <c r="N5" s="493" t="str">
+      <c r="N5" s="492" t="str">
         <f>+BALANZA!C11</f>
         <v>EQP-0046</v>
       </c>
-      <c r="O5" s="494"/>
-      <c r="P5" s="460">
+      <c r="O5" s="493"/>
+      <c r="P5" s="459">
         <f>+BALANZA!C7</f>
         <v>-3.2899999999999998E-6</v>
       </c>
-      <c r="Q5" s="461"/>
-      <c r="R5" s="495">
+      <c r="Q5" s="460"/>
+      <c r="R5" s="494">
         <f>+BALANZA!D12</f>
         <v>46132</v>
       </c>
-      <c r="S5" s="495"/>
+      <c r="S5" s="494"/>
       <c r="U5" s="79"/>
     </row>
     <row r="6" spans="1:29" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -11560,134 +11560,134 @@
     </row>
     <row r="8" spans="1:29" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="15"/>
-      <c r="B8" s="462" t="s">
+      <c r="B8" s="461" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="486" t="s">
+      <c r="C8" s="485" t="s">
         <v>3</v>
       </c>
-      <c r="D8" s="467"/>
-      <c r="E8" s="467"/>
-      <c r="F8" s="467"/>
-      <c r="G8" s="467"/>
-      <c r="H8" s="467"/>
-      <c r="I8" s="467"/>
-      <c r="J8" s="487"/>
-      <c r="K8" s="471" t="s">
+      <c r="D8" s="466"/>
+      <c r="E8" s="466"/>
+      <c r="F8" s="466"/>
+      <c r="G8" s="466"/>
+      <c r="H8" s="466"/>
+      <c r="I8" s="466"/>
+      <c r="J8" s="486"/>
+      <c r="K8" s="470" t="s">
         <v>42</v>
       </c>
-      <c r="L8" s="472"/>
-      <c r="M8" s="472"/>
-      <c r="N8" s="472"/>
-      <c r="O8" s="473"/>
-      <c r="P8" s="466" t="s">
+      <c r="L8" s="471"/>
+      <c r="M8" s="471"/>
+      <c r="N8" s="471"/>
+      <c r="O8" s="472"/>
+      <c r="P8" s="465" t="s">
         <v>18</v>
       </c>
-      <c r="Q8" s="467"/>
-      <c r="R8" s="467"/>
-      <c r="S8" s="467"/>
-      <c r="T8" s="467"/>
-      <c r="U8" s="471" t="s">
+      <c r="Q8" s="466"/>
+      <c r="R8" s="466"/>
+      <c r="S8" s="466"/>
+      <c r="T8" s="466"/>
+      <c r="U8" s="470" t="s">
         <v>43</v>
       </c>
-      <c r="V8" s="472"/>
-      <c r="W8" s="472"/>
-      <c r="X8" s="472"/>
-      <c r="Y8" s="473"/>
-      <c r="Z8" s="471" t="s">
+      <c r="V8" s="471"/>
+      <c r="W8" s="471"/>
+      <c r="X8" s="471"/>
+      <c r="Y8" s="472"/>
+      <c r="Z8" s="470" t="s">
         <v>44</v>
       </c>
-      <c r="AA8" s="472"/>
-      <c r="AB8" s="472"/>
-      <c r="AC8" s="473"/>
+      <c r="AA8" s="471"/>
+      <c r="AB8" s="471"/>
+      <c r="AC8" s="472"/>
     </row>
     <row r="9" spans="1:29" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="463"/>
-      <c r="C9" s="488"/>
-      <c r="D9" s="489"/>
-      <c r="E9" s="489"/>
-      <c r="F9" s="489"/>
-      <c r="G9" s="489"/>
-      <c r="H9" s="489"/>
-      <c r="I9" s="489"/>
-      <c r="J9" s="490"/>
-      <c r="K9" s="471"/>
-      <c r="L9" s="472"/>
-      <c r="M9" s="472"/>
-      <c r="N9" s="472"/>
-      <c r="O9" s="473"/>
-      <c r="P9" s="468"/>
-      <c r="Q9" s="469"/>
-      <c r="R9" s="469"/>
-      <c r="S9" s="469"/>
-      <c r="T9" s="469"/>
-      <c r="U9" s="471"/>
-      <c r="V9" s="472"/>
-      <c r="W9" s="472"/>
-      <c r="X9" s="472"/>
-      <c r="Y9" s="473"/>
-      <c r="Z9" s="471"/>
-      <c r="AA9" s="472"/>
-      <c r="AB9" s="472"/>
-      <c r="AC9" s="473"/>
+      <c r="B9" s="462"/>
+      <c r="C9" s="487"/>
+      <c r="D9" s="488"/>
+      <c r="E9" s="488"/>
+      <c r="F9" s="488"/>
+      <c r="G9" s="488"/>
+      <c r="H9" s="488"/>
+      <c r="I9" s="488"/>
+      <c r="J9" s="489"/>
+      <c r="K9" s="470"/>
+      <c r="L9" s="471"/>
+      <c r="M9" s="471"/>
+      <c r="N9" s="471"/>
+      <c r="O9" s="472"/>
+      <c r="P9" s="467"/>
+      <c r="Q9" s="468"/>
+      <c r="R9" s="468"/>
+      <c r="S9" s="468"/>
+      <c r="T9" s="468"/>
+      <c r="U9" s="470"/>
+      <c r="V9" s="471"/>
+      <c r="W9" s="471"/>
+      <c r="X9" s="471"/>
+      <c r="Y9" s="472"/>
+      <c r="Z9" s="470"/>
+      <c r="AA9" s="471"/>
+      <c r="AB9" s="471"/>
+      <c r="AC9" s="472"/>
     </row>
     <row r="10" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="464"/>
-      <c r="C10" s="491" t="s">
+      <c r="B10" s="463"/>
+      <c r="C10" s="490" t="s">
         <v>65</v>
       </c>
-      <c r="D10" s="491"/>
-      <c r="E10" s="491"/>
-      <c r="F10" s="455" t="s">
+      <c r="D10" s="490"/>
+      <c r="E10" s="490"/>
+      <c r="F10" s="454" t="s">
         <v>66</v>
       </c>
-      <c r="G10" s="481"/>
-      <c r="H10" s="481"/>
-      <c r="I10" s="481"/>
-      <c r="J10" s="481"/>
-      <c r="K10" s="456" t="s">
+      <c r="G10" s="480"/>
+      <c r="H10" s="480"/>
+      <c r="I10" s="480"/>
+      <c r="J10" s="480"/>
+      <c r="K10" s="455" t="s">
         <v>30</v>
       </c>
-      <c r="L10" s="454" t="s">
+      <c r="L10" s="453" t="s">
         <v>38</v>
       </c>
-      <c r="M10" s="454"/>
-      <c r="N10" s="465" t="s">
+      <c r="M10" s="453"/>
+      <c r="N10" s="464" t="s">
         <v>125</v>
       </c>
-      <c r="O10" s="474"/>
-      <c r="P10" s="470" t="s">
+      <c r="O10" s="473"/>
+      <c r="P10" s="469" t="s">
         <v>30</v>
       </c>
-      <c r="Q10" s="454" t="s">
+      <c r="Q10" s="453" t="s">
         <v>38</v>
       </c>
-      <c r="R10" s="455"/>
-      <c r="S10" s="465" t="s">
+      <c r="R10" s="454"/>
+      <c r="S10" s="464" t="s">
         <v>125</v>
       </c>
-      <c r="T10" s="425"/>
-      <c r="U10" s="456" t="s">
+      <c r="T10" s="424"/>
+      <c r="U10" s="455" t="s">
         <v>30</v>
       </c>
-      <c r="V10" s="454" t="s">
+      <c r="V10" s="453" t="s">
         <v>38</v>
       </c>
-      <c r="W10" s="454"/>
-      <c r="X10" s="465" t="s">
+      <c r="W10" s="453"/>
+      <c r="X10" s="464" t="s">
         <v>125</v>
       </c>
-      <c r="Y10" s="474"/>
-      <c r="Z10" s="456" t="s">
+      <c r="Y10" s="473"/>
+      <c r="Z10" s="455" t="s">
         <v>30</v>
       </c>
       <c r="AA10" s="80" t="s">
         <v>38</v>
       </c>
-      <c r="AB10" s="465" t="s">
+      <c r="AB10" s="464" t="s">
         <v>125</v>
       </c>
-      <c r="AC10" s="474"/>
+      <c r="AC10" s="473"/>
     </row>
     <row r="11" spans="1:29" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="81" t="s">
@@ -11717,7 +11717,7 @@
       <c r="J11" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="K11" s="456"/>
+      <c r="K11" s="455"/>
       <c r="L11" s="80" t="s">
         <v>29</v>
       </c>
@@ -11730,7 +11730,7 @@
       <c r="O11" s="163" t="s">
         <v>48</v>
       </c>
-      <c r="P11" s="470"/>
+      <c r="P11" s="469"/>
       <c r="Q11" s="80" t="s">
         <v>29</v>
       </c>
@@ -11743,7 +11743,7 @@
       <c r="T11" s="67" t="s">
         <v>48</v>
       </c>
-      <c r="U11" s="456"/>
+      <c r="U11" s="455"/>
       <c r="V11" s="80" t="s">
         <v>29</v>
       </c>
@@ -11756,7 +11756,7 @@
       <c r="Y11" s="166" t="s">
         <v>48</v>
       </c>
-      <c r="Z11" s="456"/>
+      <c r="Z11" s="455"/>
       <c r="AA11" s="80" t="s">
         <v>41</v>
       </c>
@@ -12441,10 +12441,10 @@
     </row>
     <row r="18" spans="1:31" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="18"/>
-      <c r="B18" s="484" t="s">
+      <c r="B18" s="483" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="485"/>
+      <c r="C18" s="484"/>
       <c r="D18" s="92">
         <f>SUM(D12:D17)</f>
         <v>0</v>
@@ -12490,16 +12490,16 @@
     </row>
     <row r="19" spans="1:31" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="18"/>
-      <c r="B19" s="484" t="s">
+      <c r="B19" s="483" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="485"/>
+      <c r="C19" s="484"/>
       <c r="D19" s="36" t="e">
         <f>+IF(AND(COUNTA(E12)=1,E12&gt;5),B12,IF(AND(COUNTA(E13)=1,E13&gt;5),B13,IF(AND(COUNTA(E14)=1,E14&gt;5),B14,IF(AND(COUNTA(E15)=1,E15&gt;5),B15,IF(AND(COUNTA(E16)=1,E16&gt;5),B16,IF(AND(COUNTA(E17)=1,E17&gt;5),B17))))))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E19" s="458"/>
-      <c r="F19" s="459"/>
+      <c r="E19" s="457"/>
+      <c r="F19" s="458"/>
       <c r="P19" s="59"/>
       <c r="Q19" s="59"/>
       <c r="R19" s="59"/>
@@ -12518,19 +12518,19 @@
       <c r="AE19" s="59"/>
     </row>
     <row r="20" spans="1:31" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="455" t="s">
+      <c r="B20" s="454" t="s">
         <v>62</v>
       </c>
-      <c r="C20" s="470"/>
+      <c r="C20" s="469"/>
       <c r="D20" s="93" t="e">
         <f>+IF(D19="1 1/2 in",15000,IF(D19="1 in",10000,IF(D19="3/4 in",5000,IF(D19="1/2 in",2000,IF(D19="3/8 in",1000,1000)))))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="E20" s="457" t="e">
+      <c r="E20" s="456" t="e">
         <f>+IF(D18&gt;=D20,"Cumple","No Cumple")</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F20" s="457"/>
+      <c r="F20" s="456"/>
       <c r="G20" s="35"/>
       <c r="H20" s="35"/>
       <c r="I20" s="35"/>
@@ -12832,16 +12832,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="502"/>
-      <c r="C1" s="503"/>
-      <c r="D1" s="511" t="s">
+      <c r="B1" s="501"/>
+      <c r="C1" s="502"/>
+      <c r="D1" s="510" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="512"/>
-      <c r="F1" s="512"/>
-      <c r="G1" s="512"/>
-      <c r="H1" s="512"/>
-      <c r="I1" s="513"/>
+      <c r="E1" s="511"/>
+      <c r="F1" s="511"/>
+      <c r="G1" s="511"/>
+      <c r="H1" s="511"/>
+      <c r="I1" s="512"/>
       <c r="J1" s="96" t="s">
         <v>74</v>
       </c>
@@ -12858,14 +12858,14 @@
       <c r="S1" s="97"/>
     </row>
     <row r="2" spans="2:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="504"/>
-      <c r="C2" s="505"/>
-      <c r="D2" s="514"/>
-      <c r="E2" s="515"/>
-      <c r="F2" s="515"/>
-      <c r="G2" s="515"/>
-      <c r="H2" s="515"/>
-      <c r="I2" s="516"/>
+      <c r="B2" s="503"/>
+      <c r="C2" s="504"/>
+      <c r="D2" s="513"/>
+      <c r="E2" s="514"/>
+      <c r="F2" s="514"/>
+      <c r="G2" s="514"/>
+      <c r="H2" s="514"/>
+      <c r="I2" s="515"/>
       <c r="J2" s="96" t="s">
         <v>76</v>
       </c>
@@ -12882,14 +12882,14 @@
       <c r="S2" s="97"/>
     </row>
     <row r="3" spans="2:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="504"/>
-      <c r="C3" s="505"/>
-      <c r="D3" s="514"/>
-      <c r="E3" s="515"/>
-      <c r="F3" s="515"/>
-      <c r="G3" s="515"/>
-      <c r="H3" s="515"/>
-      <c r="I3" s="516"/>
+      <c r="B3" s="503"/>
+      <c r="C3" s="504"/>
+      <c r="D3" s="513"/>
+      <c r="E3" s="514"/>
+      <c r="F3" s="514"/>
+      <c r="G3" s="514"/>
+      <c r="H3" s="514"/>
+      <c r="I3" s="515"/>
       <c r="J3" s="96" t="s">
         <v>77</v>
       </c>
@@ -12906,14 +12906,14 @@
       <c r="S3" s="97"/>
     </row>
     <row r="4" spans="2:19" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="506"/>
-      <c r="C4" s="507"/>
-      <c r="D4" s="517"/>
-      <c r="E4" s="518"/>
-      <c r="F4" s="518"/>
-      <c r="G4" s="518"/>
-      <c r="H4" s="518"/>
-      <c r="I4" s="519"/>
+      <c r="B4" s="505"/>
+      <c r="C4" s="506"/>
+      <c r="D4" s="516"/>
+      <c r="E4" s="517"/>
+      <c r="F4" s="517"/>
+      <c r="G4" s="517"/>
+      <c r="H4" s="517"/>
+      <c r="I4" s="518"/>
       <c r="J4" s="96" t="s">
         <v>78</v>
       </c>
@@ -12953,17 +12953,17 @@
       <c r="B6" s="160" t="s">
         <v>80</v>
       </c>
-      <c r="C6" s="508" t="s">
+      <c r="C6" s="507" t="s">
         <v>27</v>
       </c>
-      <c r="D6" s="509"/>
-      <c r="E6" s="509"/>
-      <c r="F6" s="509"/>
-      <c r="G6" s="509"/>
-      <c r="H6" s="509"/>
-      <c r="I6" s="509"/>
-      <c r="J6" s="509"/>
-      <c r="K6" s="510"/>
+      <c r="D6" s="508"/>
+      <c r="E6" s="508"/>
+      <c r="F6" s="508"/>
+      <c r="G6" s="508"/>
+      <c r="H6" s="508"/>
+      <c r="I6" s="508"/>
+      <c r="J6" s="508"/>
+      <c r="K6" s="509"/>
       <c r="L6" s="97"/>
       <c r="M6" s="97"/>
       <c r="N6" s="97"/>
@@ -12977,17 +12977,17 @@
       <c r="B7" s="160" t="s">
         <v>81</v>
       </c>
-      <c r="C7" s="508" t="s">
+      <c r="C7" s="507" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="509"/>
-      <c r="E7" s="509"/>
-      <c r="F7" s="509"/>
-      <c r="G7" s="509"/>
-      <c r="H7" s="509"/>
-      <c r="I7" s="509"/>
-      <c r="J7" s="509"/>
-      <c r="K7" s="510"/>
+      <c r="D7" s="508"/>
+      <c r="E7" s="508"/>
+      <c r="F7" s="508"/>
+      <c r="G7" s="508"/>
+      <c r="H7" s="508"/>
+      <c r="I7" s="508"/>
+      <c r="J7" s="508"/>
+      <c r="K7" s="509"/>
       <c r="L7" s="97"/>
       <c r="M7" s="97"/>
       <c r="N7" s="97"/>
@@ -13001,17 +13001,17 @@
       <c r="B8" s="160" t="s">
         <v>82</v>
       </c>
-      <c r="C8" s="508" t="s">
+      <c r="C8" s="507" t="s">
         <v>83</v>
       </c>
-      <c r="D8" s="509"/>
-      <c r="E8" s="509"/>
-      <c r="F8" s="509"/>
-      <c r="G8" s="509"/>
-      <c r="H8" s="509"/>
-      <c r="I8" s="509"/>
-      <c r="J8" s="509"/>
-      <c r="K8" s="510"/>
+      <c r="D8" s="508"/>
+      <c r="E8" s="508"/>
+      <c r="F8" s="508"/>
+      <c r="G8" s="508"/>
+      <c r="H8" s="508"/>
+      <c r="I8" s="508"/>
+      <c r="J8" s="508"/>
+      <c r="K8" s="509"/>
       <c r="L8" s="97"/>
       <c r="M8" s="97"/>
       <c r="N8" s="97"/>
@@ -13025,17 +13025,17 @@
       <c r="B9" s="161" t="s">
         <v>84</v>
       </c>
-      <c r="C9" s="508" t="s">
+      <c r="C9" s="507" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="509"/>
-      <c r="E9" s="509"/>
-      <c r="F9" s="509"/>
-      <c r="G9" s="509"/>
-      <c r="H9" s="509"/>
-      <c r="I9" s="509"/>
-      <c r="J9" s="509"/>
-      <c r="K9" s="510"/>
+      <c r="D9" s="508"/>
+      <c r="E9" s="508"/>
+      <c r="F9" s="508"/>
+      <c r="G9" s="508"/>
+      <c r="H9" s="508"/>
+      <c r="I9" s="508"/>
+      <c r="J9" s="508"/>
+      <c r="K9" s="509"/>
       <c r="L9" s="97"/>
       <c r="M9" s="97"/>
       <c r="N9" s="97"/>
@@ -13364,56 +13364,56 @@
       <c r="S24" s="97"/>
     </row>
     <row r="25" spans="1:39" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="498" t="s">
+      <c r="B25" s="497" t="s">
         <v>131</v>
       </c>
-      <c r="C25" s="499"/>
-      <c r="D25" s="499"/>
-      <c r="E25" s="499"/>
-      <c r="F25" s="499"/>
-      <c r="G25" s="499"/>
-      <c r="H25" s="499"/>
-      <c r="I25" s="500"/>
-      <c r="J25" s="498" t="s">
+      <c r="C25" s="498"/>
+      <c r="D25" s="498"/>
+      <c r="E25" s="498"/>
+      <c r="F25" s="498"/>
+      <c r="G25" s="498"/>
+      <c r="H25" s="498"/>
+      <c r="I25" s="499"/>
+      <c r="J25" s="497" t="s">
         <v>130</v>
       </c>
-      <c r="K25" s="499"/>
-      <c r="L25" s="499"/>
-      <c r="M25" s="499"/>
-      <c r="N25" s="500"/>
-      <c r="O25" s="498" t="s">
+      <c r="K25" s="498"/>
+      <c r="L25" s="498"/>
+      <c r="M25" s="498"/>
+      <c r="N25" s="499"/>
+      <c r="O25" s="497" t="s">
         <v>155</v>
       </c>
-      <c r="P25" s="499"/>
-      <c r="Q25" s="499"/>
-      <c r="R25" s="499"/>
-      <c r="S25" s="500"/>
-      <c r="T25" s="498" t="s">
+      <c r="P25" s="498"/>
+      <c r="Q25" s="498"/>
+      <c r="R25" s="498"/>
+      <c r="S25" s="499"/>
+      <c r="T25" s="497" t="s">
         <v>132</v>
       </c>
-      <c r="U25" s="499"/>
-      <c r="V25" s="499"/>
-      <c r="W25" s="499"/>
-      <c r="X25" s="500"/>
-      <c r="Y25" s="498" t="s">
+      <c r="U25" s="498"/>
+      <c r="V25" s="498"/>
+      <c r="W25" s="498"/>
+      <c r="X25" s="499"/>
+      <c r="Y25" s="497" t="s">
         <v>133</v>
       </c>
-      <c r="Z25" s="499"/>
-      <c r="AA25" s="499"/>
-      <c r="AB25" s="499"/>
-      <c r="AC25" s="500"/>
-      <c r="AD25" s="498" t="s">
+      <c r="Z25" s="498"/>
+      <c r="AA25" s="498"/>
+      <c r="AB25" s="498"/>
+      <c r="AC25" s="499"/>
+      <c r="AD25" s="497" t="s">
         <v>134</v>
       </c>
-      <c r="AE25" s="499"/>
-      <c r="AF25" s="499"/>
-      <c r="AG25" s="499"/>
-      <c r="AH25" s="500"/>
-      <c r="AJ25" s="501" t="s">
+      <c r="AE25" s="498"/>
+      <c r="AF25" s="498"/>
+      <c r="AG25" s="498"/>
+      <c r="AH25" s="499"/>
+      <c r="AJ25" s="500" t="s">
         <v>110</v>
       </c>
-      <c r="AK25" s="501"/>
-      <c r="AL25" s="501"/>
+      <c r="AK25" s="500"/>
+      <c r="AL25" s="500"/>
     </row>
     <row r="26" spans="1:39" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="197" t="s">
@@ -15615,56 +15615,56 @@
       <c r="S49" s="97"/>
     </row>
     <row r="50" spans="2:39" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="498" t="s">
+      <c r="B50" s="497" t="s">
         <v>131</v>
       </c>
-      <c r="C50" s="499"/>
-      <c r="D50" s="499"/>
-      <c r="E50" s="499"/>
-      <c r="F50" s="499"/>
-      <c r="G50" s="499"/>
-      <c r="H50" s="499"/>
-      <c r="I50" s="500"/>
-      <c r="J50" s="498" t="s">
+      <c r="C50" s="498"/>
+      <c r="D50" s="498"/>
+      <c r="E50" s="498"/>
+      <c r="F50" s="498"/>
+      <c r="G50" s="498"/>
+      <c r="H50" s="498"/>
+      <c r="I50" s="499"/>
+      <c r="J50" s="497" t="s">
         <v>130</v>
       </c>
-      <c r="K50" s="499"/>
-      <c r="L50" s="499"/>
-      <c r="M50" s="499"/>
-      <c r="N50" s="500"/>
-      <c r="O50" s="498" t="s">
+      <c r="K50" s="498"/>
+      <c r="L50" s="498"/>
+      <c r="M50" s="498"/>
+      <c r="N50" s="499"/>
+      <c r="O50" s="497" t="s">
         <v>155</v>
       </c>
-      <c r="P50" s="499"/>
-      <c r="Q50" s="499"/>
-      <c r="R50" s="499"/>
-      <c r="S50" s="500"/>
-      <c r="T50" s="498" t="s">
+      <c r="P50" s="498"/>
+      <c r="Q50" s="498"/>
+      <c r="R50" s="498"/>
+      <c r="S50" s="499"/>
+      <c r="T50" s="497" t="s">
         <v>132</v>
       </c>
-      <c r="U50" s="499"/>
-      <c r="V50" s="499"/>
-      <c r="W50" s="499"/>
-      <c r="X50" s="500"/>
-      <c r="Y50" s="498" t="s">
+      <c r="U50" s="498"/>
+      <c r="V50" s="498"/>
+      <c r="W50" s="498"/>
+      <c r="X50" s="499"/>
+      <c r="Y50" s="497" t="s">
         <v>133</v>
       </c>
-      <c r="Z50" s="499"/>
-      <c r="AA50" s="499"/>
-      <c r="AB50" s="499"/>
-      <c r="AC50" s="500"/>
-      <c r="AD50" s="498" t="s">
+      <c r="Z50" s="498"/>
+      <c r="AA50" s="498"/>
+      <c r="AB50" s="498"/>
+      <c r="AC50" s="499"/>
+      <c r="AD50" s="497" t="s">
         <v>134</v>
       </c>
-      <c r="AE50" s="499"/>
-      <c r="AF50" s="499"/>
-      <c r="AG50" s="499"/>
-      <c r="AH50" s="500"/>
-      <c r="AJ50" s="501" t="s">
+      <c r="AE50" s="498"/>
+      <c r="AF50" s="498"/>
+      <c r="AG50" s="498"/>
+      <c r="AH50" s="499"/>
+      <c r="AJ50" s="500" t="s">
         <v>110</v>
       </c>
-      <c r="AK50" s="501"/>
-      <c r="AL50" s="501"/>
+      <c r="AK50" s="500"/>
+      <c r="AL50" s="500"/>
     </row>
     <row r="51" spans="2:39" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="197" t="s">
@@ -17854,56 +17854,56 @@
       <c r="S74" s="97"/>
     </row>
     <row r="75" spans="2:38" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B75" s="498" t="s">
+      <c r="B75" s="497" t="s">
         <v>131</v>
       </c>
-      <c r="C75" s="499"/>
-      <c r="D75" s="499"/>
-      <c r="E75" s="499"/>
-      <c r="F75" s="499"/>
-      <c r="G75" s="499"/>
-      <c r="H75" s="499"/>
-      <c r="I75" s="500"/>
-      <c r="J75" s="498" t="s">
+      <c r="C75" s="498"/>
+      <c r="D75" s="498"/>
+      <c r="E75" s="498"/>
+      <c r="F75" s="498"/>
+      <c r="G75" s="498"/>
+      <c r="H75" s="498"/>
+      <c r="I75" s="499"/>
+      <c r="J75" s="497" t="s">
         <v>130</v>
       </c>
-      <c r="K75" s="499"/>
-      <c r="L75" s="499"/>
-      <c r="M75" s="499"/>
-      <c r="N75" s="500"/>
-      <c r="O75" s="498" t="s">
+      <c r="K75" s="498"/>
+      <c r="L75" s="498"/>
+      <c r="M75" s="498"/>
+      <c r="N75" s="499"/>
+      <c r="O75" s="497" t="s">
         <v>155</v>
       </c>
-      <c r="P75" s="499"/>
-      <c r="Q75" s="499"/>
-      <c r="R75" s="499"/>
-      <c r="S75" s="500"/>
-      <c r="T75" s="498" t="s">
+      <c r="P75" s="498"/>
+      <c r="Q75" s="498"/>
+      <c r="R75" s="498"/>
+      <c r="S75" s="499"/>
+      <c r="T75" s="497" t="s">
         <v>132</v>
       </c>
-      <c r="U75" s="499"/>
-      <c r="V75" s="499"/>
-      <c r="W75" s="499"/>
-      <c r="X75" s="500"/>
-      <c r="Y75" s="498" t="s">
+      <c r="U75" s="498"/>
+      <c r="V75" s="498"/>
+      <c r="W75" s="498"/>
+      <c r="X75" s="499"/>
+      <c r="Y75" s="497" t="s">
         <v>133</v>
       </c>
-      <c r="Z75" s="499"/>
-      <c r="AA75" s="499"/>
-      <c r="AB75" s="499"/>
-      <c r="AC75" s="500"/>
-      <c r="AD75" s="498" t="s">
+      <c r="Z75" s="498"/>
+      <c r="AA75" s="498"/>
+      <c r="AB75" s="498"/>
+      <c r="AC75" s="499"/>
+      <c r="AD75" s="497" t="s">
         <v>134</v>
       </c>
-      <c r="AE75" s="499"/>
-      <c r="AF75" s="499"/>
-      <c r="AG75" s="499"/>
-      <c r="AH75" s="500"/>
-      <c r="AJ75" s="501" t="s">
+      <c r="AE75" s="498"/>
+      <c r="AF75" s="498"/>
+      <c r="AG75" s="498"/>
+      <c r="AH75" s="499"/>
+      <c r="AJ75" s="500" t="s">
         <v>110</v>
       </c>
-      <c r="AK75" s="501"/>
-      <c r="AL75" s="501"/>
+      <c r="AK75" s="500"/>
+      <c r="AL75" s="500"/>
     </row>
     <row r="76" spans="2:38" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B76" s="197" t="s">
@@ -20093,56 +20093,56 @@
       <c r="S99" s="97"/>
     </row>
     <row r="100" spans="2:39" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B100" s="498" t="s">
+      <c r="B100" s="497" t="s">
         <v>131</v>
       </c>
-      <c r="C100" s="499"/>
-      <c r="D100" s="499"/>
-      <c r="E100" s="499"/>
-      <c r="F100" s="499"/>
-      <c r="G100" s="499"/>
-      <c r="H100" s="499"/>
-      <c r="I100" s="500"/>
-      <c r="J100" s="498" t="s">
+      <c r="C100" s="498"/>
+      <c r="D100" s="498"/>
+      <c r="E100" s="498"/>
+      <c r="F100" s="498"/>
+      <c r="G100" s="498"/>
+      <c r="H100" s="498"/>
+      <c r="I100" s="499"/>
+      <c r="J100" s="497" t="s">
         <v>130</v>
       </c>
-      <c r="K100" s="499"/>
-      <c r="L100" s="499"/>
-      <c r="M100" s="499"/>
-      <c r="N100" s="500"/>
-      <c r="O100" s="498" t="s">
+      <c r="K100" s="498"/>
+      <c r="L100" s="498"/>
+      <c r="M100" s="498"/>
+      <c r="N100" s="499"/>
+      <c r="O100" s="497" t="s">
         <v>155</v>
       </c>
-      <c r="P100" s="499"/>
-      <c r="Q100" s="499"/>
-      <c r="R100" s="499"/>
-      <c r="S100" s="500"/>
-      <c r="T100" s="498" t="s">
+      <c r="P100" s="498"/>
+      <c r="Q100" s="498"/>
+      <c r="R100" s="498"/>
+      <c r="S100" s="499"/>
+      <c r="T100" s="497" t="s">
         <v>132</v>
       </c>
-      <c r="U100" s="499"/>
-      <c r="V100" s="499"/>
-      <c r="W100" s="499"/>
-      <c r="X100" s="500"/>
-      <c r="Y100" s="498" t="s">
+      <c r="U100" s="498"/>
+      <c r="V100" s="498"/>
+      <c r="W100" s="498"/>
+      <c r="X100" s="499"/>
+      <c r="Y100" s="497" t="s">
         <v>133</v>
       </c>
-      <c r="Z100" s="499"/>
-      <c r="AA100" s="499"/>
-      <c r="AB100" s="499"/>
-      <c r="AC100" s="500"/>
-      <c r="AD100" s="498" t="s">
+      <c r="Z100" s="498"/>
+      <c r="AA100" s="498"/>
+      <c r="AB100" s="498"/>
+      <c r="AC100" s="499"/>
+      <c r="AD100" s="497" t="s">
         <v>134</v>
       </c>
-      <c r="AE100" s="499"/>
-      <c r="AF100" s="499"/>
-      <c r="AG100" s="499"/>
-      <c r="AH100" s="500"/>
-      <c r="AJ100" s="501" t="s">
+      <c r="AE100" s="498"/>
+      <c r="AF100" s="498"/>
+      <c r="AG100" s="498"/>
+      <c r="AH100" s="499"/>
+      <c r="AJ100" s="500" t="s">
         <v>110</v>
       </c>
-      <c r="AK100" s="501"/>
-      <c r="AL100" s="501"/>
+      <c r="AK100" s="500"/>
+      <c r="AL100" s="500"/>
     </row>
     <row r="101" spans="2:39" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B101" s="197" t="s">
@@ -22383,19 +22383,19 @@
       <c r="B126" s="324" t="s">
         <v>234</v>
       </c>
-      <c r="C126" s="520" t="s">
+      <c r="C126" s="519" t="s">
         <v>235</v>
       </c>
-      <c r="D126" s="521"/>
+      <c r="D126" s="520"/>
       <c r="E126" s="325"/>
-      <c r="F126" s="522" t="s">
+      <c r="F126" s="521" t="s">
         <v>236</v>
       </c>
-      <c r="G126" s="523"/>
-      <c r="H126" s="524" t="s">
+      <c r="G126" s="522"/>
+      <c r="H126" s="523" t="s">
         <v>237</v>
       </c>
-      <c r="I126" s="525"/>
+      <c r="I126" s="524"/>
       <c r="J126" s="312"/>
       <c r="K126" s="97"/>
       <c r="L126" s="97"/>
@@ -22461,19 +22461,19 @@
       <c r="B128" s="326" t="s">
         <v>238</v>
       </c>
-      <c r="C128" s="526">
+      <c r="C128" s="525">
         <v>45604</v>
       </c>
-      <c r="D128" s="527"/>
+      <c r="D128" s="526"/>
       <c r="E128" s="312"/>
-      <c r="F128" s="528" t="s">
+      <c r="F128" s="527" t="s">
         <v>239</v>
       </c>
-      <c r="G128" s="529"/>
-      <c r="H128" s="526">
+      <c r="G128" s="528"/>
+      <c r="H128" s="525">
         <v>45605</v>
       </c>
-      <c r="I128" s="527"/>
+      <c r="I128" s="526"/>
       <c r="J128" s="312"/>
       <c r="K128" s="97"/>
       <c r="L128" s="97"/>
@@ -40946,14 +40946,14 @@
     </row>
     <row r="2" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="97"/>
-      <c r="B2" s="530" t="s">
+      <c r="B2" s="529" t="s">
         <v>113</v>
       </c>
-      <c r="C2" s="531"/>
-      <c r="D2" s="531"/>
-      <c r="E2" s="531"/>
-      <c r="F2" s="531"/>
-      <c r="G2" s="531"/>
+      <c r="C2" s="530"/>
+      <c r="D2" s="530"/>
+      <c r="E2" s="530"/>
+      <c r="F2" s="530"/>
+      <c r="G2" s="530"/>
       <c r="H2" s="97"/>
       <c r="I2" s="97"/>
       <c r="J2" s="97"/>
@@ -41007,8 +41007,8 @@
       <c r="F6" s="97"/>
       <c r="G6" s="97"/>
       <c r="H6" s="97"/>
-      <c r="I6" s="532"/>
-      <c r="J6" s="531"/>
+      <c r="I6" s="531"/>
+      <c r="J6" s="530"/>
       <c r="K6" s="97"/>
     </row>
     <row r="7" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -42917,72 +42917,72 @@
       <c r="W6" s="108"/>
     </row>
     <row r="7" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="533" t="s">
+      <c r="A7" s="328" t="s">
         <v>240</v>
       </c>
-      <c r="B7" s="534">
+      <c r="B7" s="532">
         <v>3.4833333333333327E-2</v>
       </c>
-      <c r="C7" s="534"/>
-      <c r="D7" s="534"/>
-      <c r="G7" s="533" t="s">
+      <c r="C7" s="532"/>
+      <c r="D7" s="532"/>
+      <c r="G7" s="328" t="s">
         <v>240</v>
       </c>
-      <c r="H7" s="534">
+      <c r="H7" s="532">
         <v>1.4749999999999954E-3</v>
       </c>
-      <c r="I7" s="534"/>
-      <c r="J7" s="534"/>
-      <c r="M7" s="533" t="s">
+      <c r="I7" s="532"/>
+      <c r="J7" s="532"/>
+      <c r="M7" s="328" t="s">
         <v>240</v>
       </c>
-      <c r="N7" s="534">
+      <c r="N7" s="532">
         <v>2.8333333333333335E-3</v>
       </c>
-      <c r="O7" s="534"/>
-      <c r="P7" s="534"/>
-      <c r="S7" s="533" t="s">
+      <c r="O7" s="532"/>
+      <c r="P7" s="532"/>
+      <c r="S7" s="328" t="s">
         <v>240</v>
       </c>
-      <c r="T7" s="534">
+      <c r="T7" s="532">
         <v>1.35</v>
       </c>
-      <c r="U7" s="534"/>
-      <c r="V7" s="534"/>
+      <c r="U7" s="532"/>
+      <c r="V7" s="532"/>
     </row>
     <row r="8" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="533" t="s">
+      <c r="A8" s="328" t="s">
         <v>241</v>
       </c>
-      <c r="B8" s="535">
+      <c r="B8" s="533">
         <v>9.9999999999696968E-4</v>
       </c>
-      <c r="C8" s="535"/>
-      <c r="D8" s="535"/>
-      <c r="G8" s="533" t="s">
+      <c r="C8" s="533"/>
+      <c r="D8" s="533"/>
+      <c r="G8" s="328" t="s">
         <v>241</v>
       </c>
-      <c r="H8" s="535">
+      <c r="H8" s="533">
         <v>2.3333333333173337E-4</v>
       </c>
-      <c r="I8" s="535"/>
-      <c r="J8" s="535"/>
-      <c r="M8" s="533" t="s">
+      <c r="I8" s="533"/>
+      <c r="J8" s="533"/>
+      <c r="M8" s="328" t="s">
         <v>241</v>
       </c>
-      <c r="N8" s="535">
+      <c r="N8" s="533">
         <v>3.3333333333333164E-4</v>
       </c>
-      <c r="O8" s="535"/>
-      <c r="P8" s="535"/>
-      <c r="S8" s="533" t="s">
+      <c r="O8" s="533"/>
+      <c r="P8" s="533"/>
+      <c r="S8" s="328" t="s">
         <v>241</v>
       </c>
-      <c r="T8" s="535">
+      <c r="T8" s="533">
         <v>0.9</v>
       </c>
-      <c r="U8" s="535"/>
-      <c r="V8" s="535"/>
+      <c r="U8" s="533"/>
+      <c r="V8" s="533"/>
     </row>
     <row r="9" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="10" spans="1:23" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>